<commit_message>
Updated example scenario and figures
</commit_message>
<xml_diff>
--- a/data/scenarios/example_org_circ.xlsx
+++ b/data/scenarios/example_org_circ.xlsx
@@ -1,10 +1,11 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
-  <workbookPr filterPrivacy="1" defaultThemeVersion="164011"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28623"/>
+  <workbookPr filterPrivacy="1"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{28BAE003-BE4D-4216-BCD8-506D76E50C25}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="10410" tabRatio="746"/>
+    <workbookView xWindow="-38520" yWindow="-120" windowWidth="38640" windowHeight="21120" tabRatio="746" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Regions" sheetId="11" r:id="rId1"/>
@@ -17,10 +18,21 @@
     <sheet name="WasteAndCircularity" sheetId="3" r:id="rId8"/>
     <sheet name="PlantNutrientMgmt" sheetId="4" r:id="rId9"/>
   </sheets>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
     </ext>
   </extLst>
 </workbook>
@@ -515,7 +527,7 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.0"/>
   </numFmts>
@@ -704,26 +716,21 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="35">
+  <cellXfs count="28">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="164" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -744,24 +751,22 @@
     <xf numFmtId="164" fontId="7" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="1" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Percent" xfId="1" builtinId="5"/>
+    <cellStyle name="Per cent" xfId="1" builtinId="5"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -1038,7 +1043,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:M110"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
@@ -1086,7 +1091,7 @@
       </c>
     </row>
     <row r="4" spans="1:13">
-      <c r="K4" s="7" t="s">
+      <c r="K4" s="5" t="s">
         <v>153</v>
       </c>
     </row>
@@ -1106,17 +1111,17 @@
       <c r="F5" t="s">
         <v>36</v>
       </c>
-      <c r="G5" s="5">
+      <c r="G5" s="4">
         <v>0</v>
       </c>
-      <c r="H5" s="5">
+      <c r="H5" s="4">
         <f>K5*$L$3</f>
         <v>255.94738467494699</v>
       </c>
-      <c r="K5" s="5">
+      <c r="K5" s="4">
         <v>25594.738467494699</v>
       </c>
-      <c r="M5" s="30" t="s">
+      <c r="M5" s="24" t="s">
         <v>155</v>
       </c>
     </row>
@@ -1136,17 +1141,17 @@
       <c r="F6" t="s">
         <v>36</v>
       </c>
-      <c r="G6" s="5">
+      <c r="G6" s="4">
         <v>3.85524386673332</v>
       </c>
-      <c r="H6" s="5">
+      <c r="H6" s="4">
         <f t="shared" ref="H6:H69" si="0">K6*$L$3</f>
         <v>304.70923931982901</v>
       </c>
-      <c r="K6" s="5">
+      <c r="K6" s="4">
         <v>30470.923931982899</v>
       </c>
-      <c r="M6" s="30" t="s">
+      <c r="M6" s="24" t="s">
         <v>156</v>
       </c>
     </row>
@@ -1166,17 +1171,17 @@
       <c r="F7" t="s">
         <v>36</v>
       </c>
-      <c r="G7" s="5">
+      <c r="G7" s="4">
         <v>28.390559677419301</v>
       </c>
-      <c r="H7" s="5">
+      <c r="H7" s="4">
         <f t="shared" si="0"/>
         <v>299.953161813674</v>
       </c>
-      <c r="K7" s="5">
+      <c r="K7" s="4">
         <v>29995.316181367401</v>
       </c>
-      <c r="M7" s="30" t="s">
+      <c r="M7" s="24" t="s">
         <v>158</v>
       </c>
     </row>
@@ -1196,17 +1201,17 @@
       <c r="F8" t="s">
         <v>36</v>
       </c>
-      <c r="G8" s="5">
+      <c r="G8" s="4">
         <v>1.4568746404970101</v>
       </c>
-      <c r="H8" s="5">
+      <c r="H8" s="4">
         <f t="shared" si="0"/>
         <v>207.625598364898</v>
       </c>
-      <c r="K8" s="5">
+      <c r="K8" s="4">
         <v>20762.5598364898</v>
       </c>
-      <c r="M8" s="30" t="s">
+      <c r="M8" s="24" t="s">
         <v>159</v>
       </c>
     </row>
@@ -1226,14 +1231,14 @@
       <c r="F9" t="s">
         <v>36</v>
       </c>
-      <c r="G9" s="5">
+      <c r="G9" s="4">
         <v>3.12157615521265</v>
       </c>
-      <c r="H9" s="5">
+      <c r="H9" s="4">
         <f t="shared" si="0"/>
         <v>271.49729882110103</v>
       </c>
-      <c r="K9" s="5">
+      <c r="K9" s="4">
         <v>27149.729882110099</v>
       </c>
     </row>
@@ -1253,14 +1258,14 @@
       <c r="F10" t="s">
         <v>36</v>
       </c>
-      <c r="G10" s="5">
+      <c r="G10" s="4">
         <v>2.2833822580645098</v>
       </c>
-      <c r="H10" s="5">
+      <c r="H10" s="4">
         <f t="shared" si="0"/>
         <v>406.29728557399199</v>
       </c>
-      <c r="K10" s="5">
+      <c r="K10" s="4">
         <v>40629.728557399198</v>
       </c>
     </row>
@@ -1280,14 +1285,14 @@
       <c r="F11" t="s">
         <v>36</v>
       </c>
-      <c r="G11" s="5">
+      <c r="G11" s="4">
         <v>0</v>
       </c>
-      <c r="H11" s="5">
+      <c r="H11" s="4">
         <f t="shared" si="0"/>
         <v>292.58245666252799</v>
       </c>
-      <c r="K11" s="5">
+      <c r="K11" s="4">
         <v>29258.245666252798</v>
       </c>
     </row>
@@ -1307,14 +1312,14 @@
       <c r="F12" t="s">
         <v>36</v>
       </c>
-      <c r="G12" s="5">
+      <c r="G12" s="4">
         <v>3.33418709677419</v>
       </c>
-      <c r="H12" s="5">
+      <c r="H12" s="4">
         <f t="shared" si="0"/>
         <v>322.61307686954302</v>
       </c>
-      <c r="K12" s="5">
+      <c r="K12" s="4">
         <v>32261.3076869543</v>
       </c>
     </row>
@@ -1334,14 +1339,14 @@
       <c r="F13" t="s">
         <v>36</v>
       </c>
-      <c r="G13" s="5">
+      <c r="G13" s="4">
         <v>0</v>
       </c>
-      <c r="H13" s="5">
+      <c r="H13" s="4">
         <f t="shared" si="0"/>
         <v>149.098933268471</v>
       </c>
-      <c r="K13" s="5">
+      <c r="K13" s="4">
         <v>14909.893326847099</v>
       </c>
     </row>
@@ -1361,14 +1366,14 @@
       <c r="F14" t="s">
         <v>36</v>
       </c>
-      <c r="G14" s="5">
+      <c r="G14" s="4">
         <v>5.0568120791127803E-2</v>
       </c>
-      <c r="H14" s="5">
+      <c r="H14" s="4">
         <f t="shared" si="0"/>
         <v>108.848233566283</v>
       </c>
-      <c r="K14" s="5">
+      <c r="K14" s="4">
         <v>10884.8233566283</v>
       </c>
     </row>
@@ -1388,14 +1393,14 @@
       <c r="F15" t="s">
         <v>36</v>
       </c>
-      <c r="G15" s="5">
+      <c r="G15" s="4">
         <v>9.5731145161290296</v>
       </c>
-      <c r="H15" s="5">
+      <c r="H15" s="4">
         <f t="shared" si="0"/>
         <v>425.79028809374404</v>
       </c>
-      <c r="K15" s="5">
+      <c r="K15" s="4">
         <v>42579.028809374402</v>
       </c>
     </row>
@@ -1415,14 +1420,14 @@
       <c r="F16" t="s">
         <v>36</v>
       </c>
-      <c r="G16" s="5">
+      <c r="G16" s="4">
         <v>0</v>
       </c>
-      <c r="H16" s="5">
+      <c r="H16" s="4">
         <f t="shared" si="0"/>
         <v>273.90022763511701</v>
       </c>
-      <c r="K16" s="5">
+      <c r="K16" s="4">
         <v>27390.022763511701</v>
       </c>
     </row>
@@ -1442,14 +1447,14 @@
       <c r="F17" t="s">
         <v>36</v>
       </c>
-      <c r="G17" s="5">
+      <c r="G17" s="4">
         <v>0</v>
       </c>
-      <c r="H17" s="5">
+      <c r="H17" s="4">
         <f t="shared" si="0"/>
         <v>234.328185557002</v>
       </c>
-      <c r="K17" s="5">
+      <c r="K17" s="4">
         <v>23432.8185557002</v>
       </c>
     </row>
@@ -1469,14 +1474,14 @@
       <c r="F18" t="s">
         <v>36</v>
       </c>
-      <c r="G18" s="5">
+      <c r="G18" s="4">
         <v>5.0765967741935398</v>
       </c>
-      <c r="H18" s="5">
+      <c r="H18" s="4">
         <f t="shared" si="0"/>
         <v>319.14326572592302</v>
       </c>
-      <c r="K18" s="5">
+      <c r="K18" s="4">
         <v>31914.326572592301</v>
       </c>
     </row>
@@ -1496,14 +1501,14 @@
       <c r="F19" t="s">
         <v>36</v>
       </c>
-      <c r="G19" s="5">
+      <c r="G19" s="4">
         <v>2.9858499999999899</v>
       </c>
-      <c r="H19" s="5">
+      <c r="H19" s="4">
         <f t="shared" si="0"/>
         <v>514.10457479258196</v>
       </c>
-      <c r="K19" s="5">
+      <c r="K19" s="4">
         <v>51410.457479258199</v>
       </c>
     </row>
@@ -1523,14 +1528,14 @@
       <c r="F20" t="s">
         <v>36</v>
       </c>
-      <c r="G20" s="5">
+      <c r="G20" s="4">
         <v>5.4973532258064504</v>
       </c>
-      <c r="H20" s="5">
+      <c r="H20" s="4">
         <f t="shared" si="0"/>
         <v>444.56214437804101</v>
       </c>
-      <c r="K20" s="5">
+      <c r="K20" s="4">
         <v>44456.214437804098</v>
       </c>
     </row>
@@ -1550,14 +1555,14 @@
       <c r="F21" t="s">
         <v>36</v>
       </c>
-      <c r="G21" s="5">
+      <c r="G21" s="4">
         <v>10.3921774193548</v>
       </c>
-      <c r="H21" s="5">
+      <c r="H21" s="4">
         <f t="shared" si="0"/>
         <v>173.92603008132701</v>
       </c>
-      <c r="K21" s="5">
+      <c r="K21" s="4">
         <v>17392.603008132701</v>
       </c>
     </row>
@@ -1577,14 +1582,14 @@
       <c r="F22" t="s">
         <v>36</v>
       </c>
-      <c r="G22" s="5">
+      <c r="G22" s="4">
         <v>9.9996645161290303</v>
       </c>
-      <c r="H22" s="5">
+      <c r="H22" s="4">
         <f t="shared" si="0"/>
         <v>211.77348443123702</v>
       </c>
-      <c r="K22" s="5">
+      <c r="K22" s="4">
         <v>21177.348443123701</v>
       </c>
     </row>
@@ -1604,14 +1609,14 @@
       <c r="F23" t="s">
         <v>36</v>
       </c>
-      <c r="G23" s="5">
+      <c r="G23" s="4">
         <v>7.9666243654822297</v>
       </c>
-      <c r="H23" s="5">
+      <c r="H23" s="4">
         <f t="shared" si="0"/>
         <v>362.515526566294</v>
       </c>
-      <c r="K23" s="5">
+      <c r="K23" s="4">
         <v>36251.552656629399</v>
       </c>
     </row>
@@ -1631,14 +1636,14 @@
       <c r="F24" t="s">
         <v>36</v>
       </c>
-      <c r="G24" s="5">
+      <c r="G24" s="4">
         <v>0</v>
       </c>
-      <c r="H24" s="5">
+      <c r="H24" s="4">
         <f t="shared" si="0"/>
         <v>369.01952520574201</v>
       </c>
-      <c r="K24" s="5">
+      <c r="K24" s="4">
         <v>36901.952520574203</v>
       </c>
     </row>
@@ -1658,14 +1663,14 @@
       <c r="F25" t="s">
         <v>36</v>
       </c>
-      <c r="G25" s="5">
+      <c r="G25" s="4">
         <v>5.9847792665449498E-2</v>
       </c>
-      <c r="H25" s="5">
+      <c r="H25" s="4">
         <f t="shared" si="0"/>
         <v>109.40458549732901</v>
       </c>
-      <c r="K25" s="5">
+      <c r="K25" s="4">
         <v>10940.458549732901</v>
       </c>
     </row>
@@ -1685,14 +1690,14 @@
       <c r="F26" t="s">
         <v>36</v>
       </c>
-      <c r="G26" s="5">
+      <c r="G26" s="4">
         <v>5.6030911976997197</v>
       </c>
-      <c r="H26" s="5">
+      <c r="H26" s="4">
         <f t="shared" si="0"/>
         <v>260.75858565248103</v>
       </c>
-      <c r="K26" s="5">
+      <c r="K26" s="4">
         <v>26075.858565248102</v>
       </c>
     </row>
@@ -1712,14 +1717,14 @@
       <c r="F27" t="s">
         <v>36</v>
       </c>
-      <c r="G27" s="5">
+      <c r="G27" s="4">
         <v>19.649878857142799</v>
       </c>
-      <c r="H27" s="5">
+      <c r="H27" s="4">
         <f t="shared" si="0"/>
         <v>156.85734778602702</v>
       </c>
-      <c r="K27" s="5">
+      <c r="K27" s="4">
         <v>15685.7347786027</v>
       </c>
     </row>
@@ -1739,14 +1744,14 @@
       <c r="F28" t="s">
         <v>36</v>
       </c>
-      <c r="G28" s="5">
+      <c r="G28" s="4">
         <v>23.407983238095198</v>
       </c>
-      <c r="H28" s="5">
+      <c r="H28" s="4">
         <f t="shared" si="0"/>
         <v>233.194038082909</v>
       </c>
-      <c r="K28" s="5">
+      <c r="K28" s="4">
         <v>23319.403808290899</v>
       </c>
     </row>
@@ -1766,14 +1771,14 @@
       <c r="F29" t="s">
         <v>36</v>
       </c>
-      <c r="G29" s="5">
+      <c r="G29" s="4">
         <v>21.919931428571399</v>
       </c>
-      <c r="H29" s="5">
+      <c r="H29" s="4">
         <f t="shared" si="0"/>
         <v>159.70658457586902</v>
       </c>
-      <c r="K29" s="5">
+      <c r="K29" s="4">
         <v>15970.6584575869</v>
       </c>
     </row>
@@ -1793,14 +1798,14 @@
       <c r="F30" t="s">
         <v>36</v>
       </c>
-      <c r="G30" s="5">
+      <c r="G30" s="4">
         <v>0.198347796192821</v>
       </c>
-      <c r="H30" s="5">
+      <c r="H30" s="4">
         <f t="shared" si="0"/>
         <v>335.12959494746298</v>
       </c>
-      <c r="K30" s="5">
+      <c r="K30" s="4">
         <v>33512.959494746297</v>
       </c>
     </row>
@@ -1820,14 +1825,14 @@
       <c r="F31" t="s">
         <v>36</v>
       </c>
-      <c r="G31" s="5">
+      <c r="G31" s="4">
         <v>16.805983999999999</v>
       </c>
-      <c r="H31" s="5">
+      <c r="H31" s="4">
         <f t="shared" si="0"/>
         <v>328.196802270364</v>
       </c>
-      <c r="K31" s="5">
+      <c r="K31" s="4">
         <v>32819.680227036399</v>
       </c>
     </row>
@@ -1847,14 +1852,14 @@
       <c r="F32" t="s">
         <v>36</v>
       </c>
-      <c r="G32" s="5">
+      <c r="G32" s="4">
         <v>1.43265506464887</v>
       </c>
-      <c r="H32" s="5">
+      <c r="H32" s="4">
         <f t="shared" si="0"/>
         <v>158.12143738184702</v>
       </c>
-      <c r="K32" s="5">
+      <c r="K32" s="4">
         <v>15812.143738184701</v>
       </c>
     </row>
@@ -1874,14 +1879,14 @@
       <c r="F33" t="s">
         <v>36</v>
       </c>
-      <c r="G33" s="5">
+      <c r="G33" s="4">
         <v>13.6976716190476</v>
       </c>
-      <c r="H33" s="5">
+      <c r="H33" s="4">
         <f t="shared" si="0"/>
         <v>196.40458204037401</v>
       </c>
-      <c r="K33" s="5">
+      <c r="K33" s="4">
         <v>19640.458204037401</v>
       </c>
     </row>
@@ -1901,14 +1906,14 @@
       <c r="F34" t="s">
         <v>36</v>
       </c>
-      <c r="G34" s="5">
+      <c r="G34" s="4">
         <v>0</v>
       </c>
-      <c r="H34" s="5">
+      <c r="H34" s="4">
         <f t="shared" si="0"/>
         <v>90.780608691938596</v>
       </c>
-      <c r="K34" s="5">
+      <c r="K34" s="4">
         <v>9078.0608691938596</v>
       </c>
     </row>
@@ -1928,14 +1933,14 @@
       <c r="F35" t="s">
         <v>36</v>
       </c>
-      <c r="G35" s="5">
+      <c r="G35" s="4">
         <v>6.1342695113458996</v>
       </c>
-      <c r="H35" s="5">
+      <c r="H35" s="4">
         <f t="shared" si="0"/>
         <v>279.12440119518999</v>
       </c>
-      <c r="K35" s="5">
+      <c r="K35" s="4">
         <v>27912.440119519</v>
       </c>
     </row>
@@ -1955,14 +1960,14 @@
       <c r="F36" t="s">
         <v>36</v>
       </c>
-      <c r="G36" s="5">
+      <c r="G36" s="4">
         <v>0</v>
       </c>
-      <c r="H36" s="5">
+      <c r="H36" s="4">
         <f t="shared" si="0"/>
         <v>241.05913007931002</v>
       </c>
-      <c r="K36" s="5">
+      <c r="K36" s="4">
         <v>24105.913007931002</v>
       </c>
     </row>
@@ -1982,14 +1987,14 @@
       <c r="F37" t="s">
         <v>36</v>
       </c>
-      <c r="G37" s="5">
+      <c r="G37" s="4">
         <v>0</v>
       </c>
-      <c r="H37" s="5">
+      <c r="H37" s="4">
         <f t="shared" si="0"/>
         <v>254.411615241389</v>
       </c>
-      <c r="K37" s="5">
+      <c r="K37" s="4">
         <v>25441.161524138901</v>
       </c>
     </row>
@@ -2009,14 +2014,14 @@
       <c r="F38" t="s">
         <v>36</v>
       </c>
-      <c r="G38" s="5">
+      <c r="G38" s="4">
         <v>19.395306666666599</v>
       </c>
-      <c r="H38" s="5">
+      <c r="H38" s="4">
         <f t="shared" si="0"/>
         <v>250.19830913809099</v>
       </c>
-      <c r="K38" s="5">
+      <c r="K38" s="4">
         <v>25019.830913809099</v>
       </c>
     </row>
@@ -2036,14 +2041,14 @@
       <c r="F39" t="s">
         <v>36</v>
       </c>
-      <c r="G39" s="5">
+      <c r="G39" s="4">
         <v>0</v>
       </c>
-      <c r="H39" s="5">
+      <c r="H39" s="4">
         <f t="shared" si="0"/>
         <v>350.39342916824603</v>
       </c>
-      <c r="K39" s="5">
+      <c r="K39" s="4">
         <v>35039.3429168246</v>
       </c>
     </row>
@@ -2063,14 +2068,14 @@
       <c r="F40" t="s">
         <v>36</v>
       </c>
-      <c r="G40" s="5">
+      <c r="G40" s="4">
         <v>0</v>
       </c>
-      <c r="H40" s="5">
+      <c r="H40" s="4">
         <f t="shared" si="0"/>
         <v>125.46956607126199</v>
       </c>
-      <c r="K40" s="5">
+      <c r="K40" s="4">
         <v>12546.9566071262</v>
       </c>
     </row>
@@ -2090,14 +2095,14 @@
       <c r="F41" t="s">
         <v>36</v>
       </c>
-      <c r="G41" s="5">
+      <c r="G41" s="4">
         <v>68.060789333333304</v>
       </c>
-      <c r="H41" s="5">
+      <c r="H41" s="4">
         <f t="shared" si="0"/>
         <v>428.002241716887</v>
       </c>
-      <c r="K41" s="5">
+      <c r="K41" s="4">
         <v>42800.2241716887</v>
       </c>
     </row>
@@ -2117,14 +2122,14 @@
       <c r="F42" t="s">
         <v>36</v>
       </c>
-      <c r="G42" s="5">
+      <c r="G42" s="4">
         <v>100.45756190476099</v>
       </c>
-      <c r="H42" s="5">
+      <c r="H42" s="4">
         <f t="shared" si="0"/>
         <v>538.56653394577404</v>
       </c>
-      <c r="K42" s="5">
+      <c r="K42" s="4">
         <v>53856.653394577399</v>
       </c>
     </row>
@@ -2144,14 +2149,14 @@
       <c r="F43" t="s">
         <v>36</v>
       </c>
-      <c r="G43" s="5">
+      <c r="G43" s="4">
         <v>112.987858285714</v>
       </c>
-      <c r="H43" s="5">
+      <c r="H43" s="4">
         <f t="shared" si="0"/>
         <v>346.36805396601898</v>
       </c>
-      <c r="K43" s="5">
+      <c r="K43" s="4">
         <v>34636.8053966019</v>
       </c>
     </row>
@@ -2171,14 +2176,14 @@
       <c r="F44" t="s">
         <v>36</v>
       </c>
-      <c r="G44" s="5">
+      <c r="G44" s="4">
         <v>10.4030963132426</v>
       </c>
-      <c r="H44" s="5">
+      <c r="H44" s="4">
         <f t="shared" si="0"/>
         <v>225.14061547774503</v>
       </c>
-      <c r="K44" s="5">
+      <c r="K44" s="4">
         <v>22514.061547774501</v>
       </c>
     </row>
@@ -2198,14 +2203,14 @@
       <c r="F45" t="s">
         <v>36</v>
       </c>
-      <c r="G45" s="5">
+      <c r="G45" s="4">
         <v>0.48703902992513498</v>
       </c>
-      <c r="H45" s="5">
+      <c r="H45" s="4">
         <f t="shared" si="0"/>
         <v>265.739127238707</v>
       </c>
-      <c r="K45" s="5">
+      <c r="K45" s="4">
         <v>26573.912723870701</v>
       </c>
     </row>
@@ -2225,14 +2230,14 @@
       <c r="F46" t="s">
         <v>36</v>
       </c>
-      <c r="G46" s="5">
+      <c r="G46" s="4">
         <v>0</v>
       </c>
-      <c r="H46" s="5">
+      <c r="H46" s="4">
         <f t="shared" si="0"/>
         <v>185.842381381249</v>
       </c>
-      <c r="K46" s="5">
+      <c r="K46" s="4">
         <v>18584.2381381249</v>
       </c>
     </row>
@@ -2252,14 +2257,14 @@
       <c r="F47" t="s">
         <v>36</v>
       </c>
-      <c r="G47" s="5">
+      <c r="G47" s="4">
         <v>65.799477398392099</v>
       </c>
-      <c r="H47" s="5">
+      <c r="H47" s="4">
         <f t="shared" si="0"/>
         <v>132.010819999999</v>
       </c>
-      <c r="K47" s="5">
+      <c r="K47" s="4">
         <v>13201.0819999999</v>
       </c>
     </row>
@@ -2279,14 +2284,14 @@
       <c r="F48" t="s">
         <v>36</v>
       </c>
-      <c r="G48" s="5">
+      <c r="G48" s="4">
         <v>26.162650446065999</v>
       </c>
-      <c r="H48" s="5">
+      <c r="H48" s="4">
         <f t="shared" si="0"/>
         <v>211.02876762073402</v>
       </c>
-      <c r="K48" s="5">
+      <c r="K48" s="4">
         <v>21102.8767620734</v>
       </c>
     </row>
@@ -2306,14 +2311,14 @@
       <c r="F49" t="s">
         <v>36</v>
       </c>
-      <c r="G49" s="5">
+      <c r="G49" s="4">
         <v>4.3498798658230298</v>
       </c>
-      <c r="H49" s="5">
+      <c r="H49" s="4">
         <f t="shared" si="0"/>
         <v>66.496745122023711</v>
       </c>
-      <c r="K49" s="5">
+      <c r="K49" s="4">
         <v>6649.6745122023704</v>
       </c>
     </row>
@@ -2333,14 +2338,14 @@
       <c r="F50" t="s">
         <v>36</v>
       </c>
-      <c r="G50" s="5">
+      <c r="G50" s="4">
         <v>0</v>
       </c>
-      <c r="H50" s="5">
+      <c r="H50" s="4">
         <f t="shared" si="0"/>
         <v>75.889655445932505</v>
       </c>
-      <c r="K50" s="5">
+      <c r="K50" s="4">
         <v>7588.9655445932503</v>
       </c>
     </row>
@@ -2360,14 +2365,14 @@
       <c r="F51" t="s">
         <v>36</v>
       </c>
-      <c r="G51" s="5">
+      <c r="G51" s="4">
         <v>0.97926309520096899</v>
       </c>
-      <c r="H51" s="5">
+      <c r="H51" s="4">
         <f t="shared" si="0"/>
         <v>163.41945777951901</v>
       </c>
-      <c r="K51" s="5">
+      <c r="K51" s="4">
         <v>16341.9457779519</v>
       </c>
     </row>
@@ -2387,14 +2392,14 @@
       <c r="F52" t="s">
         <v>36</v>
       </c>
-      <c r="G52" s="5">
+      <c r="G52" s="4">
         <v>27.699412429378501</v>
       </c>
-      <c r="H52" s="5">
+      <c r="H52" s="4">
         <f t="shared" si="0"/>
         <v>472.86017038036402</v>
       </c>
-      <c r="K52" s="5">
+      <c r="K52" s="4">
         <v>47286.0170380364</v>
       </c>
     </row>
@@ -2414,14 +2419,14 @@
       <c r="F53" t="s">
         <v>36</v>
       </c>
-      <c r="G53" s="5">
+      <c r="G53" s="4">
         <v>7.4069864686597597</v>
       </c>
-      <c r="H53" s="5">
+      <c r="H53" s="4">
         <f t="shared" si="0"/>
         <v>121.105718758188</v>
       </c>
-      <c r="K53" s="5">
+      <c r="K53" s="4">
         <v>12110.5718758188</v>
       </c>
     </row>
@@ -2441,14 +2446,14 @@
       <c r="F54" t="s">
         <v>36</v>
       </c>
-      <c r="G54" s="5">
+      <c r="G54" s="4">
         <v>60.650818142207399</v>
       </c>
-      <c r="H54" s="5">
+      <c r="H54" s="4">
         <f t="shared" si="0"/>
         <v>274.57694441744701</v>
       </c>
-      <c r="K54" s="5">
+      <c r="K54" s="4">
         <v>27457.694441744701</v>
       </c>
     </row>
@@ -2468,14 +2473,14 @@
       <c r="F55" t="s">
         <v>36</v>
       </c>
-      <c r="G55" s="5">
+      <c r="G55" s="4">
         <v>234.198886227743</v>
       </c>
-      <c r="H55" s="5">
+      <c r="H55" s="4">
         <f t="shared" si="0"/>
         <v>426.32752983142501</v>
       </c>
-      <c r="K55" s="5">
+      <c r="K55" s="4">
         <v>42632.752983142498</v>
       </c>
     </row>
@@ -2495,14 +2500,14 @@
       <c r="F56" t="s">
         <v>36</v>
       </c>
-      <c r="G56" s="5">
+      <c r="G56" s="4">
         <v>175.95729233572899</v>
       </c>
-      <c r="H56" s="5">
+      <c r="H56" s="4">
         <f t="shared" si="0"/>
         <v>207.43627270073</v>
       </c>
-      <c r="K56" s="5">
+      <c r="K56" s="4">
         <v>20743.627270073001</v>
       </c>
     </row>
@@ -2522,14 +2527,14 @@
       <c r="F57" t="s">
         <v>36</v>
       </c>
-      <c r="G57" s="5">
+      <c r="G57" s="4">
         <v>430.30658760609498</v>
       </c>
-      <c r="H57" s="5">
+      <c r="H57" s="4">
         <f t="shared" si="0"/>
         <v>427.342263926155</v>
       </c>
-      <c r="K57" s="5">
+      <c r="K57" s="4">
         <v>42734.226392615499</v>
       </c>
     </row>
@@ -2549,14 +2554,14 @@
       <c r="F58" t="s">
         <v>36</v>
       </c>
-      <c r="G58" s="5">
+      <c r="G58" s="4">
         <v>68.298017007517501</v>
       </c>
-      <c r="H58" s="5">
+      <c r="H58" s="4">
         <f t="shared" si="0"/>
         <v>233.980803472708</v>
       </c>
-      <c r="K58" s="5">
+      <c r="K58" s="4">
         <v>23398.080347270799</v>
       </c>
     </row>
@@ -2576,14 +2581,14 @@
       <c r="F59" t="s">
         <v>36</v>
       </c>
-      <c r="G59" s="5">
+      <c r="G59" s="4">
         <v>171.24747479030401</v>
       </c>
-      <c r="H59" s="5">
+      <c r="H59" s="4">
         <f t="shared" si="0"/>
         <v>399.53786699256801</v>
       </c>
-      <c r="K59" s="5">
+      <c r="K59" s="4">
         <v>39953.786699256802</v>
       </c>
     </row>
@@ -2603,14 +2608,14 @@
       <c r="F60" t="s">
         <v>36</v>
       </c>
-      <c r="G60" s="5">
+      <c r="G60" s="4">
         <v>22.9929761166253</v>
       </c>
-      <c r="H60" s="5">
+      <c r="H60" s="4">
         <f t="shared" si="0"/>
         <v>150.40684926943501</v>
       </c>
-      <c r="K60" s="5">
+      <c r="K60" s="4">
         <v>15040.684926943501</v>
       </c>
     </row>
@@ -2630,14 +2635,14 @@
       <c r="F61" t="s">
         <v>36</v>
       </c>
-      <c r="G61" s="5">
+      <c r="G61" s="4">
         <v>0</v>
       </c>
-      <c r="H61" s="5">
+      <c r="H61" s="4">
         <f t="shared" si="0"/>
         <v>0.64757999999999993</v>
       </c>
-      <c r="K61" s="5">
+      <c r="K61" s="4">
         <v>64.757999999999996</v>
       </c>
     </row>
@@ -2657,14 +2662,14 @@
       <c r="F62" t="s">
         <v>36</v>
       </c>
-      <c r="G62" s="5">
+      <c r="G62" s="4">
         <v>12.4091051901664</v>
       </c>
-      <c r="H62" s="5">
+      <c r="H62" s="4">
         <f t="shared" si="0"/>
         <v>326.13707781566802</v>
       </c>
-      <c r="K62" s="5">
+      <c r="K62" s="4">
         <v>32613.707781566802</v>
       </c>
     </row>
@@ -2684,14 +2689,14 @@
       <c r="F63" t="s">
         <v>36</v>
       </c>
-      <c r="G63" s="5">
+      <c r="G63" s="4">
         <v>106.282471783687</v>
       </c>
-      <c r="H63" s="5">
+      <c r="H63" s="4">
         <f t="shared" si="0"/>
         <v>233.025101390282</v>
       </c>
-      <c r="K63" s="5">
+      <c r="K63" s="4">
         <v>23302.5101390282</v>
       </c>
     </row>
@@ -2711,14 +2716,14 @@
       <c r="F64" t="s">
         <v>36</v>
       </c>
-      <c r="G64" s="5">
+      <c r="G64" s="4">
         <v>33.7829500714153</v>
       </c>
-      <c r="H64" s="5">
+      <c r="H64" s="4">
         <f t="shared" si="0"/>
         <v>66.036650140690895</v>
       </c>
-      <c r="K64" s="5">
+      <c r="K64" s="4">
         <v>6603.6650140690899</v>
       </c>
     </row>
@@ -2738,14 +2743,14 @@
       <c r="F65" t="s">
         <v>36</v>
       </c>
-      <c r="G65" s="5">
+      <c r="G65" s="4">
         <v>0</v>
       </c>
-      <c r="H65" s="5">
+      <c r="H65" s="4">
         <f t="shared" si="0"/>
         <v>130.09066393646401</v>
       </c>
-      <c r="K65" s="5">
+      <c r="K65" s="4">
         <v>13009.066393646401</v>
       </c>
     </row>
@@ -2765,14 +2770,14 @@
       <c r="F66" t="s">
         <v>36</v>
       </c>
-      <c r="G66" s="5">
+      <c r="G66" s="4">
         <v>28.51</v>
       </c>
-      <c r="H66" s="5">
+      <c r="H66" s="4">
         <f t="shared" si="0"/>
         <v>197.836471547087</v>
       </c>
-      <c r="K66" s="5">
+      <c r="K66" s="4">
         <v>19783.647154708699</v>
       </c>
     </row>
@@ -2792,14 +2797,14 @@
       <c r="F67" t="s">
         <v>36</v>
       </c>
-      <c r="G67" s="5">
+      <c r="G67" s="4">
         <v>3.0161733742290799</v>
       </c>
-      <c r="H67" s="5">
+      <c r="H67" s="4">
         <f t="shared" si="0"/>
         <v>178.78732824512699</v>
       </c>
-      <c r="K67" s="5">
+      <c r="K67" s="4">
         <v>17878.732824512699</v>
       </c>
     </row>
@@ -2819,14 +2824,14 @@
       <c r="F68" t="s">
         <v>36</v>
       </c>
-      <c r="G68" s="5">
+      <c r="G68" s="4">
         <v>9.6434617202012003</v>
       </c>
-      <c r="H68" s="5">
+      <c r="H68" s="4">
         <f t="shared" si="0"/>
         <v>233.03889196620901</v>
       </c>
-      <c r="K68" s="5">
+      <c r="K68" s="4">
         <v>23303.889196620901</v>
       </c>
     </row>
@@ -2846,14 +2851,14 @@
       <c r="F69" t="s">
         <v>36</v>
       </c>
-      <c r="G69" s="5">
+      <c r="G69" s="4">
         <v>0</v>
       </c>
-      <c r="H69" s="5">
+      <c r="H69" s="4">
         <f t="shared" si="0"/>
         <v>102.29819999999999</v>
       </c>
-      <c r="K69" s="5">
+      <c r="K69" s="4">
         <v>10229.82</v>
       </c>
     </row>
@@ -2873,14 +2878,14 @@
       <c r="F70" t="s">
         <v>36</v>
       </c>
-      <c r="G70" s="5">
+      <c r="G70" s="4">
         <v>0</v>
       </c>
-      <c r="H70" s="5">
+      <c r="H70" s="4">
         <f t="shared" ref="H70:H110" si="1">K70*$L$3</f>
         <v>27.000019999999999</v>
       </c>
-      <c r="K70" s="5">
+      <c r="K70" s="4">
         <v>2700.002</v>
       </c>
     </row>
@@ -2900,14 +2905,14 @@
       <c r="F71" t="s">
         <v>36</v>
       </c>
-      <c r="G71" s="5">
+      <c r="G71" s="4">
         <v>0</v>
       </c>
-      <c r="H71" s="5">
+      <c r="H71" s="4">
         <f t="shared" si="1"/>
         <v>31.1934421990481</v>
       </c>
-      <c r="K71" s="5">
+      <c r="K71" s="4">
         <v>3119.34421990481</v>
       </c>
     </row>
@@ -2927,14 +2932,14 @@
       <c r="F72" t="s">
         <v>36</v>
       </c>
-      <c r="G72" s="5">
+      <c r="G72" s="4">
         <v>0.30171428571428499</v>
       </c>
-      <c r="H72" s="5">
+      <c r="H72" s="4">
         <f t="shared" si="1"/>
         <v>183.66356435679501</v>
       </c>
-      <c r="K72" s="5">
+      <c r="K72" s="4">
         <v>18366.3564356795</v>
       </c>
     </row>
@@ -2954,14 +2959,14 @@
       <c r="F73" t="s">
         <v>36</v>
       </c>
-      <c r="G73" s="5">
+      <c r="G73" s="4">
         <v>0</v>
       </c>
-      <c r="H73" s="5">
+      <c r="H73" s="4">
         <f t="shared" si="1"/>
         <v>94.752857737488497</v>
       </c>
-      <c r="K73" s="5">
+      <c r="K73" s="4">
         <v>9475.2857737488503</v>
       </c>
     </row>
@@ -2981,14 +2986,14 @@
       <c r="F74" t="s">
         <v>36</v>
       </c>
-      <c r="G74" s="5">
+      <c r="G74" s="4">
         <v>0</v>
       </c>
-      <c r="H74" s="5">
+      <c r="H74" s="4">
         <f t="shared" si="1"/>
         <v>174.66265625076602</v>
       </c>
-      <c r="K74" s="5">
+      <c r="K74" s="4">
         <v>17466.265625076601</v>
       </c>
     </row>
@@ -3008,14 +3013,14 @@
       <c r="F75" t="s">
         <v>36</v>
       </c>
-      <c r="G75" s="5">
+      <c r="G75" s="4">
         <v>1.1792942624009599</v>
       </c>
-      <c r="H75" s="5">
+      <c r="H75" s="4">
         <f t="shared" si="1"/>
         <v>171.914706892287</v>
       </c>
-      <c r="K75" s="5">
+      <c r="K75" s="4">
         <v>17191.470689228699</v>
       </c>
     </row>
@@ -3035,14 +3040,14 @@
       <c r="F76" t="s">
         <v>36</v>
       </c>
-      <c r="G76" s="5">
+      <c r="G76" s="4">
         <v>0</v>
       </c>
-      <c r="H76" s="5">
+      <c r="H76" s="4">
         <f t="shared" si="1"/>
         <v>32.804659999999998</v>
       </c>
-      <c r="K76" s="5">
+      <c r="K76" s="4">
         <v>3280.4659999999999</v>
       </c>
     </row>
@@ -3062,14 +3067,14 @@
       <c r="F77" t="s">
         <v>36</v>
       </c>
-      <c r="G77" s="5">
+      <c r="G77" s="4">
         <v>0</v>
       </c>
-      <c r="H77" s="5">
+      <c r="H77" s="4">
         <f t="shared" si="1"/>
         <v>3.1147000000000005</v>
       </c>
-      <c r="K77" s="5">
+      <c r="K77" s="4">
         <v>311.47000000000003</v>
       </c>
     </row>
@@ -3089,14 +3094,14 @@
       <c r="F78" t="s">
         <v>36</v>
       </c>
-      <c r="G78" s="5">
+      <c r="G78" s="4">
         <v>0.59030541775922296</v>
       </c>
-      <c r="H78" s="5">
+      <c r="H78" s="4">
         <f t="shared" si="1"/>
         <v>194.19755947327201</v>
       </c>
-      <c r="K78" s="5">
+      <c r="K78" s="4">
         <v>19419.755947327201</v>
       </c>
     </row>
@@ -3116,14 +3121,14 @@
       <c r="F79" t="s">
         <v>36</v>
       </c>
-      <c r="G79" s="5">
+      <c r="G79" s="4">
         <v>0</v>
       </c>
-      <c r="H79" s="5">
+      <c r="H79" s="4">
         <f t="shared" si="1"/>
         <v>103.89191289291601</v>
       </c>
-      <c r="K79" s="5">
+      <c r="K79" s="4">
         <v>10389.191289291601</v>
       </c>
     </row>
@@ -3143,14 +3148,14 @@
       <c r="F80" t="s">
         <v>36</v>
       </c>
-      <c r="G80" s="5">
+      <c r="G80" s="4">
         <v>0</v>
       </c>
-      <c r="H80" s="5">
+      <c r="H80" s="4">
         <f t="shared" si="1"/>
         <v>2.92936</v>
       </c>
-      <c r="K80" s="5">
+      <c r="K80" s="4">
         <v>292.93599999999998</v>
       </c>
     </row>
@@ -3170,14 +3175,14 @@
       <c r="F81" t="s">
         <v>36</v>
       </c>
-      <c r="G81" s="5">
+      <c r="G81" s="4">
         <v>0</v>
       </c>
-      <c r="H81" s="5">
+      <c r="H81" s="4">
         <f t="shared" si="1"/>
         <v>18.154107322534703</v>
       </c>
-      <c r="K81" s="5">
+      <c r="K81" s="4">
         <v>1815.4107322534701</v>
       </c>
     </row>
@@ -3197,14 +3202,14 @@
       <c r="F82" t="s">
         <v>36</v>
       </c>
-      <c r="G82" s="5">
+      <c r="G82" s="4">
         <v>86.191315172757598</v>
       </c>
-      <c r="H82" s="5">
+      <c r="H82" s="4">
         <f t="shared" si="1"/>
         <v>538.81435189539502</v>
       </c>
-      <c r="K82" s="5">
+      <c r="K82" s="4">
         <v>53881.435189539501</v>
       </c>
     </row>
@@ -3224,14 +3229,14 @@
       <c r="F83" t="s">
         <v>36</v>
       </c>
-      <c r="G83" s="5">
+      <c r="G83" s="4">
         <v>51.547613856836101</v>
       </c>
-      <c r="H83" s="5">
+      <c r="H83" s="4">
         <f t="shared" si="1"/>
         <v>216.36378444708501</v>
       </c>
-      <c r="K83" s="5">
+      <c r="K83" s="4">
         <v>21636.378444708502</v>
       </c>
     </row>
@@ -3251,14 +3256,14 @@
       <c r="F84" t="s">
         <v>36</v>
       </c>
-      <c r="G84" s="5">
+      <c r="G84" s="4">
         <v>174.451971174862</v>
       </c>
-      <c r="H84" s="5">
+      <c r="H84" s="4">
         <f t="shared" si="1"/>
         <v>508.52337939894102</v>
       </c>
-      <c r="K84" s="5">
+      <c r="K84" s="4">
         <v>50852.337939894103</v>
       </c>
     </row>
@@ -3278,14 +3283,14 @@
       <c r="F85" t="s">
         <v>36</v>
       </c>
-      <c r="G85" s="5">
+      <c r="G85" s="4">
         <v>12.2023910226289</v>
       </c>
-      <c r="H85" s="5">
+      <c r="H85" s="4">
         <f t="shared" si="1"/>
         <v>119.15531535771899</v>
       </c>
-      <c r="K85" s="5">
+      <c r="K85" s="4">
         <v>11915.531535771899</v>
       </c>
     </row>
@@ -3305,14 +3310,14 @@
       <c r="F86" t="s">
         <v>36</v>
       </c>
-      <c r="G86" s="5">
+      <c r="G86" s="4">
         <v>27.514925098187501</v>
       </c>
-      <c r="H86" s="5">
+      <c r="H86" s="4">
         <f t="shared" si="1"/>
         <v>359.50401688626903</v>
       </c>
-      <c r="K86" s="5">
+      <c r="K86" s="4">
         <v>35950.401688626902</v>
       </c>
     </row>
@@ -3332,14 +3337,14 @@
       <c r="F87" t="s">
         <v>36</v>
       </c>
-      <c r="G87" s="5">
+      <c r="G87" s="4">
         <v>28.865765763490401</v>
       </c>
-      <c r="H87" s="5">
+      <c r="H87" s="4">
         <f t="shared" si="1"/>
         <v>354.95392859352006</v>
       </c>
-      <c r="K87" s="5">
+      <c r="K87" s="4">
         <v>35495.392859352003</v>
       </c>
     </row>
@@ -3359,14 +3364,14 @@
       <c r="F88" t="s">
         <v>36</v>
       </c>
-      <c r="G88" s="5">
+      <c r="G88" s="4">
         <v>37.582730679716597</v>
       </c>
-      <c r="H88" s="5">
+      <c r="H88" s="4">
         <f t="shared" si="1"/>
         <v>246.06402332780502</v>
       </c>
-      <c r="K88" s="5">
+      <c r="K88" s="4">
         <v>24606.402332780501</v>
       </c>
     </row>
@@ -3386,14 +3391,14 @@
       <c r="F89" t="s">
         <v>36</v>
       </c>
-      <c r="G89" s="5">
+      <c r="G89" s="4">
         <v>22.0288663629415</v>
       </c>
-      <c r="H89" s="5">
+      <c r="H89" s="4">
         <f t="shared" si="1"/>
         <v>341.51816767079799</v>
       </c>
-      <c r="K89" s="5">
+      <c r="K89" s="4">
         <v>34151.816767079799</v>
       </c>
     </row>
@@ -3413,14 +3418,14 @@
       <c r="F90" t="s">
         <v>36</v>
       </c>
-      <c r="G90" s="5">
+      <c r="G90" s="4">
         <v>0</v>
       </c>
-      <c r="H90" s="5">
+      <c r="H90" s="4">
         <f t="shared" si="1"/>
         <v>111.71078595133801</v>
       </c>
-      <c r="K90" s="5">
+      <c r="K90" s="4">
         <v>11171.0785951338</v>
       </c>
     </row>
@@ -3440,14 +3445,14 @@
       <c r="F91" t="s">
         <v>36</v>
       </c>
-      <c r="G91" s="5">
+      <c r="G91" s="4">
         <v>0</v>
       </c>
-      <c r="H91" s="5">
+      <c r="H91" s="4">
         <f t="shared" si="1"/>
         <v>153.469847481431</v>
       </c>
-      <c r="K91" s="5">
+      <c r="K91" s="4">
         <v>15346.984748143101</v>
       </c>
     </row>
@@ -3467,14 +3472,14 @@
       <c r="F92" t="s">
         <v>36</v>
       </c>
-      <c r="G92" s="5">
+      <c r="G92" s="4">
         <v>3.09395637198622</v>
       </c>
-      <c r="H92" s="5">
+      <c r="H92" s="4">
         <f t="shared" si="1"/>
         <v>459.86800376061302</v>
       </c>
-      <c r="K92" s="5">
+      <c r="K92" s="4">
         <v>45986.800376061299</v>
       </c>
     </row>
@@ -3494,14 +3499,14 @@
       <c r="F93" t="s">
         <v>36</v>
       </c>
-      <c r="G93" s="5">
+      <c r="G93" s="4">
         <v>0</v>
       </c>
-      <c r="H93" s="5">
+      <c r="H93" s="4">
         <f t="shared" si="1"/>
         <v>476.12173363926797</v>
       </c>
-      <c r="K93" s="5">
+      <c r="K93" s="4">
         <v>47612.173363926799</v>
       </c>
     </row>
@@ -3521,14 +3526,14 @@
       <c r="F94" t="s">
         <v>36</v>
       </c>
-      <c r="G94" s="5">
+      <c r="G94" s="4">
         <v>3.5611492537313398</v>
       </c>
-      <c r="H94" s="5">
+      <c r="H94" s="4">
         <f t="shared" si="1"/>
         <v>438.47014697697904</v>
       </c>
-      <c r="K94" s="5">
+      <c r="K94" s="4">
         <v>43847.014697697901</v>
       </c>
     </row>
@@ -3548,14 +3553,14 @@
       <c r="F95" t="s">
         <v>36</v>
       </c>
-      <c r="G95" s="5">
+      <c r="G95" s="4">
         <v>0.37522538636098002</v>
       </c>
-      <c r="H95" s="5">
+      <c r="H95" s="4">
         <f t="shared" si="1"/>
         <v>226.94207518871602</v>
       </c>
-      <c r="K95" s="5">
+      <c r="K95" s="4">
         <v>22694.207518871601</v>
       </c>
     </row>
@@ -3575,14 +3580,14 @@
       <c r="F96" t="s">
         <v>36</v>
       </c>
-      <c r="G96" s="5">
+      <c r="G96" s="4">
         <v>0</v>
       </c>
-      <c r="H96" s="5">
+      <c r="H96" s="4">
         <f t="shared" si="1"/>
         <v>148.988240504911</v>
       </c>
-      <c r="K96" s="5">
+      <c r="K96" s="4">
         <v>14898.824050491099</v>
       </c>
     </row>
@@ -3602,14 +3607,14 @@
       <c r="F97" t="s">
         <v>36</v>
       </c>
-      <c r="G97" s="5">
+      <c r="G97" s="4">
         <v>0</v>
       </c>
-      <c r="H97" s="5">
+      <c r="H97" s="4">
         <f t="shared" si="1"/>
         <v>229.21768902455901</v>
       </c>
-      <c r="K97" s="5">
+      <c r="K97" s="4">
         <v>22921.7689024559</v>
       </c>
     </row>
@@ -3629,14 +3634,14 @@
       <c r="F98" t="s">
         <v>36</v>
       </c>
-      <c r="G98" s="5">
+      <c r="G98" s="4">
         <v>0.24597514250772301</v>
       </c>
-      <c r="H98" s="5">
+      <c r="H98" s="4">
         <f t="shared" si="1"/>
         <v>210.38200616856699</v>
       </c>
-      <c r="K98" s="5">
+      <c r="K98" s="4">
         <v>21038.200616856699</v>
       </c>
     </row>
@@ -3656,14 +3661,14 @@
       <c r="F99" t="s">
         <v>36</v>
       </c>
-      <c r="G99" s="5">
+      <c r="G99" s="4">
         <v>0</v>
       </c>
-      <c r="H99" s="5">
+      <c r="H99" s="4">
         <f t="shared" si="1"/>
         <v>307.22668098460798</v>
       </c>
-      <c r="K99" s="5">
+      <c r="K99" s="4">
         <v>30722.668098460799</v>
       </c>
     </row>
@@ -3683,14 +3688,14 @@
       <c r="F100" t="s">
         <v>36</v>
       </c>
-      <c r="G100" s="5">
+      <c r="G100" s="4">
         <v>0.119259259259259</v>
       </c>
-      <c r="H100" s="5">
+      <c r="H100" s="4">
         <f t="shared" si="1"/>
         <v>193.70152851346199</v>
       </c>
-      <c r="K100" s="5">
+      <c r="K100" s="4">
         <v>19370.1528513462</v>
       </c>
     </row>
@@ -3710,14 +3715,14 @@
       <c r="F101" t="s">
         <v>36</v>
       </c>
-      <c r="G101" s="5">
+      <c r="G101" s="4">
         <v>0</v>
       </c>
-      <c r="H101" s="5">
+      <c r="H101" s="4">
         <f t="shared" si="1"/>
         <v>101.614774238858</v>
       </c>
-      <c r="K101" s="5">
+      <c r="K101" s="4">
         <v>10161.477423885801</v>
       </c>
     </row>
@@ -3737,14 +3742,14 @@
       <c r="F102" t="s">
         <v>36</v>
       </c>
-      <c r="G102" s="5">
+      <c r="G102" s="4">
         <v>0.23198026054161699</v>
       </c>
-      <c r="H102" s="5">
+      <c r="H102" s="4">
         <f t="shared" si="1"/>
         <v>379.58382471254299</v>
       </c>
-      <c r="K102" s="5">
+      <c r="K102" s="4">
         <v>37958.382471254299</v>
       </c>
     </row>
@@ -3764,14 +3769,14 @@
       <c r="F103" t="s">
         <v>36</v>
       </c>
-      <c r="G103" s="5">
+      <c r="G103" s="4">
         <v>0</v>
       </c>
-      <c r="H103" s="5">
+      <c r="H103" s="4">
         <f t="shared" si="1"/>
         <v>274.53578179206499</v>
       </c>
-      <c r="K103" s="5">
+      <c r="K103" s="4">
         <v>27453.578179206499</v>
       </c>
     </row>
@@ -3791,14 +3796,14 @@
       <c r="F104" t="s">
         <v>36</v>
       </c>
-      <c r="G104" s="5">
+      <c r="G104" s="4">
         <v>0</v>
       </c>
-      <c r="H104" s="5">
+      <c r="H104" s="4">
         <f t="shared" si="1"/>
         <v>125.557666536157</v>
       </c>
-      <c r="K104" s="5">
+      <c r="K104" s="4">
         <v>12555.766653615699</v>
       </c>
     </row>
@@ -3818,14 +3823,14 @@
       <c r="F105" t="s">
         <v>36</v>
       </c>
-      <c r="G105" s="5">
+      <c r="G105" s="4">
         <v>0</v>
       </c>
-      <c r="H105" s="5">
+      <c r="H105" s="4">
         <f t="shared" si="1"/>
         <v>140.741755149456</v>
       </c>
-      <c r="K105" s="5">
+      <c r="K105" s="4">
         <v>14074.1755149456</v>
       </c>
     </row>
@@ -3845,14 +3850,14 @@
       <c r="F106" t="s">
         <v>36</v>
       </c>
-      <c r="G106" s="5">
+      <c r="G106" s="4">
         <v>0</v>
       </c>
-      <c r="H106" s="5">
+      <c r="H106" s="4">
         <f t="shared" si="1"/>
         <v>310.85539079934597</v>
       </c>
-      <c r="K106" s="5">
+      <c r="K106" s="4">
         <v>31085.539079934599</v>
       </c>
     </row>
@@ -3872,14 +3877,14 @@
       <c r="F107" t="s">
         <v>36</v>
       </c>
-      <c r="G107" s="5">
+      <c r="G107" s="4">
         <v>0</v>
       </c>
-      <c r="H107" s="5">
+      <c r="H107" s="4">
         <f t="shared" si="1"/>
         <v>161.485810125559</v>
       </c>
-      <c r="K107" s="5">
+      <c r="K107" s="4">
         <v>16148.5810125559</v>
       </c>
     </row>
@@ -3899,14 +3904,14 @@
       <c r="F108" t="s">
         <v>36</v>
       </c>
-      <c r="G108" s="5">
+      <c r="G108" s="4">
         <v>2.06691937765205</v>
       </c>
-      <c r="H108" s="5">
+      <c r="H108" s="4">
         <f t="shared" si="1"/>
         <v>193.19351790153999</v>
       </c>
-      <c r="K108" s="5">
+      <c r="K108" s="4">
         <v>19319.351790154</v>
       </c>
     </row>
@@ -3926,14 +3931,14 @@
       <c r="F109" t="s">
         <v>36</v>
       </c>
-      <c r="G109" s="5">
+      <c r="G109" s="4">
         <v>64.281776520509098</v>
       </c>
-      <c r="H109" s="5">
+      <c r="H109" s="4">
         <f t="shared" si="1"/>
         <v>468.317185661547</v>
       </c>
-      <c r="K109" s="5">
+      <c r="K109" s="4">
         <v>46831.718566154697</v>
       </c>
     </row>
@@ -3953,14 +3958,14 @@
       <c r="F110" t="s">
         <v>36</v>
       </c>
-      <c r="G110" s="5">
+      <c r="G110" s="4">
         <v>0</v>
       </c>
-      <c r="H110" s="5">
+      <c r="H110" s="4">
         <f t="shared" si="1"/>
         <v>190.29927643691099</v>
       </c>
-      <c r="K110" s="5">
+      <c r="K110" s="4">
         <v>19029.927643691099</v>
       </c>
     </row>
@@ -3971,7 +3976,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:S82"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
@@ -4017,13 +4022,7 @@
     <row r="2" spans="1:19">
       <c r="D2" s="1"/>
       <c r="E2" s="1"/>
-      <c r="G2" s="2"/>
-      <c r="H2" s="2"/>
-      <c r="I2" s="3"/>
-      <c r="P2" s="13"/>
-      <c r="Q2" s="13"/>
-      <c r="R2" s="13"/>
-      <c r="S2" s="13"/>
+      <c r="I2" s="2"/>
     </row>
     <row r="3" spans="1:19">
       <c r="B3" t="s">
@@ -4034,19 +4033,17 @@
       <c r="F3" t="s">
         <v>41</v>
       </c>
-      <c r="G3" s="2" t="s">
+      <c r="G3" t="s">
         <v>10</v>
       </c>
-      <c r="H3" s="2">
-        <v>1</v>
-      </c>
-      <c r="I3" s="3">
+      <c r="H3">
+        <v>1</v>
+      </c>
+      <c r="I3" s="2">
         <v>1.39</v>
       </c>
-      <c r="P3" s="13"/>
-      <c r="Q3" s="14"/>
-      <c r="R3" s="14"/>
-      <c r="S3" s="13"/>
+      <c r="Q3" s="1"/>
+      <c r="R3" s="1"/>
     </row>
     <row r="4" spans="1:19">
       <c r="B4" t="s">
@@ -4057,19 +4054,17 @@
       <c r="F4" t="s">
         <v>41</v>
       </c>
-      <c r="G4" s="2" t="s">
+      <c r="G4" t="s">
         <v>10</v>
       </c>
-      <c r="H4" s="2">
-        <v>1</v>
-      </c>
-      <c r="I4" s="3">
+      <c r="H4">
+        <v>1</v>
+      </c>
+      <c r="I4" s="2">
         <v>1.58</v>
       </c>
-      <c r="P4" s="13"/>
-      <c r="Q4" s="14"/>
-      <c r="R4" s="14"/>
-      <c r="S4" s="13"/>
+      <c r="Q4" s="1"/>
+      <c r="R4" s="1"/>
     </row>
     <row r="5" spans="1:19">
       <c r="B5" t="s">
@@ -4080,30 +4075,24 @@
       <c r="F5" t="s">
         <v>41</v>
       </c>
-      <c r="G5" s="2" t="s">
+      <c r="G5" t="s">
         <v>10</v>
       </c>
-      <c r="H5" s="2">
-        <v>1</v>
-      </c>
-      <c r="I5" s="3">
+      <c r="H5">
+        <v>1</v>
+      </c>
+      <c r="I5" s="2">
         <v>1.58</v>
       </c>
-      <c r="P5" s="13"/>
-      <c r="Q5" s="14"/>
-      <c r="R5" s="14"/>
-      <c r="S5" s="13"/>
+      <c r="Q5" s="1"/>
+      <c r="R5" s="1"/>
     </row>
     <row r="6" spans="1:19">
       <c r="D6" s="1"/>
       <c r="E6" s="1"/>
-      <c r="G6" s="2"/>
-      <c r="H6" s="2"/>
-      <c r="I6" s="3"/>
-      <c r="P6" s="13"/>
-      <c r="Q6" s="14"/>
-      <c r="R6" s="14"/>
-      <c r="S6" s="13"/>
+      <c r="I6" s="2"/>
+      <c r="Q6" s="1"/>
+      <c r="R6" s="1"/>
     </row>
     <row r="7" spans="1:19">
       <c r="B7" t="s">
@@ -4114,19 +4103,17 @@
       <c r="F7" t="s">
         <v>41</v>
       </c>
-      <c r="G7" s="2" t="s">
+      <c r="G7" t="s">
         <v>10</v>
       </c>
-      <c r="H7" s="2">
-        <v>1</v>
-      </c>
-      <c r="I7" s="3">
+      <c r="H7">
+        <v>1</v>
+      </c>
+      <c r="I7" s="2">
         <v>0.85</v>
       </c>
-      <c r="P7" s="13"/>
-      <c r="Q7" s="14"/>
-      <c r="R7" s="14"/>
-      <c r="S7" s="13"/>
+      <c r="Q7" s="1"/>
+      <c r="R7" s="1"/>
     </row>
     <row r="8" spans="1:19">
       <c r="A8" t="s">
@@ -4140,33 +4127,27 @@
       <c r="F8" t="s">
         <v>41</v>
       </c>
-      <c r="G8" s="2" t="s">
+      <c r="G8" t="s">
         <v>10</v>
       </c>
-      <c r="H8" s="2">
-        <v>1</v>
-      </c>
-      <c r="I8" s="3">
+      <c r="H8">
+        <v>1</v>
+      </c>
+      <c r="I8" s="2">
         <v>0.65</v>
       </c>
-      <c r="M8" s="28" t="s">
+      <c r="M8" s="22" t="s">
         <v>88</v>
       </c>
-      <c r="P8" s="13"/>
-      <c r="Q8" s="14"/>
-      <c r="R8" s="14"/>
-      <c r="S8" s="13"/>
+      <c r="Q8" s="1"/>
+      <c r="R8" s="1"/>
     </row>
     <row r="9" spans="1:19">
       <c r="D9" s="1"/>
       <c r="E9" s="1"/>
-      <c r="G9" s="2"/>
-      <c r="H9" s="2"/>
-      <c r="I9" s="3"/>
-      <c r="P9" s="13"/>
-      <c r="Q9" s="14"/>
-      <c r="R9" s="14"/>
-      <c r="S9" s="13"/>
+      <c r="I9" s="2"/>
+      <c r="Q9" s="1"/>
+      <c r="R9" s="1"/>
     </row>
     <row r="10" spans="1:19">
       <c r="A10" t="s">
@@ -4175,19 +4156,18 @@
       <c r="F10" t="s">
         <v>41</v>
       </c>
-      <c r="G10" s="2" t="s">
+      <c r="G10" t="s">
         <v>10</v>
       </c>
       <c r="H10">
         <v>1</v>
       </c>
-      <c r="I10" s="3">
+      <c r="I10" s="2">
         <v>0.59</v>
       </c>
-      <c r="P10" s="13"/>
-      <c r="Q10" s="15"/>
-      <c r="R10" s="15"/>
-      <c r="S10" s="16"/>
+      <c r="Q10" s="6"/>
+      <c r="R10" s="6"/>
+      <c r="S10" s="11"/>
     </row>
     <row r="11" spans="1:19">
       <c r="A11" t="s">
@@ -4196,19 +4176,18 @@
       <c r="F11" t="s">
         <v>41</v>
       </c>
-      <c r="G11" s="2" t="s">
+      <c r="G11" t="s">
         <v>10</v>
       </c>
       <c r="H11">
         <v>1</v>
       </c>
-      <c r="I11" s="3">
+      <c r="I11" s="2">
         <v>0.59</v>
       </c>
-      <c r="P11" s="13"/>
-      <c r="Q11" s="15"/>
-      <c r="R11" s="15"/>
-      <c r="S11" s="16"/>
+      <c r="Q11" s="6"/>
+      <c r="R11" s="6"/>
+      <c r="S11" s="11"/>
     </row>
     <row r="12" spans="1:19">
       <c r="A12" t="s">
@@ -4217,19 +4196,18 @@
       <c r="F12" t="s">
         <v>41</v>
       </c>
-      <c r="G12" s="2" t="s">
+      <c r="G12" t="s">
         <v>10</v>
       </c>
       <c r="H12">
         <v>1</v>
       </c>
-      <c r="I12" s="3">
+      <c r="I12" s="2">
         <v>0.59</v>
       </c>
-      <c r="P12" s="13"/>
-      <c r="Q12" s="15"/>
-      <c r="R12" s="15"/>
-      <c r="S12" s="16"/>
+      <c r="Q12" s="6"/>
+      <c r="R12" s="6"/>
+      <c r="S12" s="11"/>
     </row>
     <row r="13" spans="1:19">
       <c r="A13" t="s">
@@ -4238,19 +4216,17 @@
       <c r="F13" t="s">
         <v>41</v>
       </c>
-      <c r="G13" s="2" t="s">
+      <c r="G13" t="s">
         <v>10</v>
       </c>
       <c r="H13">
         <v>1</v>
       </c>
-      <c r="I13" s="3">
+      <c r="I13" s="2">
         <v>0.86</v>
       </c>
-      <c r="P13" s="13"/>
-      <c r="Q13" s="15"/>
-      <c r="R13" s="15"/>
-      <c r="S13" s="13"/>
+      <c r="Q13" s="6"/>
+      <c r="R13" s="6"/>
     </row>
     <row r="14" spans="1:19">
       <c r="A14" t="s">
@@ -4259,27 +4235,20 @@
       <c r="F14" t="s">
         <v>41</v>
       </c>
-      <c r="G14" s="2" t="s">
+      <c r="G14" t="s">
         <v>10</v>
       </c>
       <c r="H14">
         <v>1</v>
       </c>
-      <c r="I14" s="3">
+      <c r="I14" s="2">
         <v>0.5</v>
       </c>
-      <c r="P14" s="13"/>
-      <c r="Q14" s="15"/>
-      <c r="R14" s="15"/>
-      <c r="S14" s="13"/>
+      <c r="Q14" s="6"/>
+      <c r="R14" s="6"/>
     </row>
     <row r="15" spans="1:19">
-      <c r="G15" s="2"/>
-      <c r="I15" s="9"/>
-      <c r="P15" s="13"/>
-      <c r="Q15" s="13"/>
-      <c r="R15" s="13"/>
-      <c r="S15" s="13"/>
+      <c r="I15" s="7"/>
     </row>
     <row r="16" spans="1:19">
       <c r="A16" t="s">
@@ -4288,81 +4257,70 @@
       <c r="F16" t="s">
         <v>41</v>
       </c>
-      <c r="G16" s="2" t="s">
+      <c r="G16" t="s">
         <v>36</v>
       </c>
       <c r="H16">
         <v>4.5</v>
       </c>
-      <c r="I16" s="9">
+      <c r="I16" s="7">
         <f>H16*$K$17</f>
         <v>15.525</v>
       </c>
-      <c r="P16" s="13"/>
-      <c r="Q16" s="15"/>
-      <c r="R16" s="15"/>
-      <c r="S16" s="17"/>
+      <c r="Q16" s="6"/>
+      <c r="R16" s="6"/>
+      <c r="S16" s="12"/>
     </row>
     <row r="17" spans="1:19">
-      <c r="A17" s="8" t="s">
+      <c r="A17" s="6" t="s">
         <v>43</v>
       </c>
       <c r="F17" t="s">
         <v>41</v>
       </c>
-      <c r="G17" s="2" t="s">
-        <v>36</v>
-      </c>
-      <c r="H17" s="2">
+      <c r="G17" t="s">
+        <v>36</v>
+      </c>
+      <c r="H17">
         <v>0</v>
       </c>
-      <c r="I17" s="9">
+      <c r="I17" s="7">
         <f>I16</f>
         <v>15.525</v>
       </c>
       <c r="K17">
         <v>3.45</v>
       </c>
-      <c r="P17" s="13"/>
-      <c r="Q17" s="15"/>
-      <c r="R17" s="15"/>
-      <c r="S17" s="13"/>
+      <c r="Q17" s="6"/>
+      <c r="R17" s="6"/>
     </row>
     <row r="18" spans="1:19">
-      <c r="A18" s="8" t="s">
+      <c r="A18" s="6" t="s">
         <v>44</v>
       </c>
       <c r="F18" t="s">
         <v>41</v>
       </c>
-      <c r="G18" s="2" t="s">
-        <v>36</v>
-      </c>
-      <c r="H18" s="2">
+      <c r="G18" t="s">
+        <v>36</v>
+      </c>
+      <c r="H18">
         <v>0.7</v>
       </c>
-      <c r="I18" s="9">
+      <c r="I18" s="7">
         <f>H18*$K$17</f>
         <v>2.415</v>
       </c>
-      <c r="K18" s="11">
+      <c r="K18" s="9">
         <f>(SUM(I16:I18)-SUM(H16:H18))/SUM(H16:H18)</f>
         <v>5.4355769230769235</v>
       </c>
-      <c r="P18" s="13"/>
-      <c r="Q18" s="15"/>
-      <c r="R18" s="15"/>
-      <c r="S18" s="13"/>
+      <c r="Q18" s="6"/>
+      <c r="R18" s="6"/>
     </row>
     <row r="19" spans="1:19">
-      <c r="A19" s="8"/>
-      <c r="G19" s="2"/>
-      <c r="H19" s="2"/>
-      <c r="I19" s="9"/>
-      <c r="P19" s="13"/>
-      <c r="Q19" s="13"/>
-      <c r="R19" s="13"/>
-      <c r="S19" s="13"/>
+      <c r="A19" s="6"/>
+      <c r="I19" s="7"/>
     </row>
     <row r="20" spans="1:19">
       <c r="A20" t="s">
@@ -4371,28 +4329,25 @@
       <c r="F20" t="s">
         <v>41</v>
       </c>
-      <c r="G20" s="2" t="s">
+      <c r="G20" t="s">
         <v>10</v>
       </c>
-      <c r="H20" s="10">
-        <v>1</v>
-      </c>
-      <c r="I20" s="3">
+      <c r="H20" s="8">
+        <v>1</v>
+      </c>
+      <c r="I20" s="2">
         <v>1.05</v>
       </c>
-      <c r="P20" s="13"/>
-      <c r="Q20" s="15"/>
-      <c r="R20" s="15"/>
-      <c r="S20" s="16"/>
+      <c r="Q20" s="6"/>
+      <c r="R20" s="6"/>
+      <c r="S20" s="11"/>
     </row>
     <row r="21" spans="1:19">
-      <c r="G21" s="2"/>
-      <c r="H21" s="10"/>
-      <c r="I21" s="3"/>
-      <c r="P21" s="13"/>
-      <c r="Q21" s="15"/>
-      <c r="R21" s="15"/>
-      <c r="S21" s="16"/>
+      <c r="H21" s="8"/>
+      <c r="I21" s="2"/>
+      <c r="Q21" s="6"/>
+      <c r="R21" s="6"/>
+      <c r="S21" s="11"/>
     </row>
     <row r="22" spans="1:19">
       <c r="A22" t="s">
@@ -4401,62 +4356,54 @@
       <c r="F22" t="s">
         <v>41</v>
       </c>
-      <c r="G22" s="2" t="s">
+      <c r="G22" t="s">
         <v>10</v>
       </c>
-      <c r="H22" s="10">
-        <v>1</v>
-      </c>
-      <c r="I22" s="3">
+      <c r="H22" s="8">
+        <v>1</v>
+      </c>
+      <c r="I22" s="2">
         <v>0.34</v>
       </c>
-      <c r="P22" s="13"/>
-      <c r="Q22" s="15"/>
-      <c r="R22" s="15"/>
-      <c r="S22" s="16"/>
+      <c r="Q22" s="6"/>
+      <c r="R22" s="6"/>
+      <c r="S22" s="11"/>
     </row>
     <row r="23" spans="1:19">
-      <c r="G23" s="2"/>
-      <c r="H23" s="10"/>
-      <c r="I23" s="3"/>
-      <c r="P23" s="13"/>
-      <c r="Q23" s="15"/>
-      <c r="R23" s="15"/>
-      <c r="S23" s="16"/>
+      <c r="H23" s="8"/>
+      <c r="I23" s="2"/>
+      <c r="Q23" s="6"/>
+      <c r="R23" s="6"/>
+      <c r="S23" s="11"/>
     </row>
     <row r="24" spans="1:19">
-      <c r="A24" s="8"/>
+      <c r="A24" s="6"/>
       <c r="E24" t="s">
         <v>89</v>
       </c>
       <c r="F24" t="s">
         <v>90</v>
       </c>
-      <c r="G24" s="2" t="s">
+      <c r="G24" t="s">
         <v>10</v>
       </c>
-      <c r="H24" s="2">
-        <v>1</v>
-      </c>
-      <c r="I24" s="3">
+      <c r="H24">
+        <v>1</v>
+      </c>
+      <c r="I24" s="2">
         <v>0.5</v>
       </c>
-      <c r="P24" s="13"/>
-      <c r="Q24" s="34"/>
-      <c r="R24" s="34"/>
-      <c r="S24" s="13"/>
+      <c r="Q24" s="27"/>
+      <c r="R24" s="27"/>
     </row>
     <row r="25" spans="1:19">
-      <c r="A25" s="8"/>
-      <c r="H25" s="2"/>
-      <c r="I25" s="3"/>
-      <c r="P25" s="13"/>
-      <c r="Q25" s="18"/>
-      <c r="R25" s="18"/>
-      <c r="S25" s="13"/>
+      <c r="A25" s="6"/>
+      <c r="I25" s="2"/>
+      <c r="Q25" s="13"/>
+      <c r="R25" s="13"/>
     </row>
     <row r="26" spans="1:19">
-      <c r="A26" s="4" t="s">
+      <c r="A26" s="3" t="s">
         <v>21</v>
       </c>
       <c r="B26" t="s">
@@ -4474,23 +4421,15 @@
       <c r="H26">
         <v>0</v>
       </c>
-      <c r="I26" s="5">
+      <c r="I26" s="4">
         <v>1000000</v>
       </c>
-      <c r="K26" s="27" t="s">
+      <c r="K26" s="21" t="s">
         <v>25</v>
       </c>
-      <c r="P26" s="13"/>
-      <c r="Q26" s="13"/>
-      <c r="R26" s="13"/>
-      <c r="S26" s="13"/>
     </row>
     <row r="27" spans="1:19">
-      <c r="K27" s="29"/>
-      <c r="P27" s="13"/>
-      <c r="Q27" s="13"/>
-      <c r="R27" s="13"/>
-      <c r="S27" s="13"/>
+      <c r="K27" s="23"/>
     </row>
     <row r="28" spans="1:19">
       <c r="A28" t="s">
@@ -4511,20 +4450,16 @@
       <c r="H28">
         <v>0</v>
       </c>
-      <c r="I28" s="5">
+      <c r="I28" s="4">
         <f>558250*0.3</f>
         <v>167475</v>
       </c>
-      <c r="K28" s="29" t="s">
+      <c r="K28" s="23" t="s">
         <v>87</v>
       </c>
-      <c r="M28" s="28" t="s">
+      <c r="M28" s="22" t="s">
         <v>147</v>
       </c>
-      <c r="P28" s="13"/>
-      <c r="Q28" s="13"/>
-      <c r="R28" s="13"/>
-      <c r="S28" s="13"/>
     </row>
     <row r="29" spans="1:19">
       <c r="A29" t="s">
@@ -4545,17 +4480,13 @@
       <c r="H29">
         <v>0</v>
       </c>
-      <c r="I29" s="5">
+      <c r="I29" s="4">
         <f>518197*0.25</f>
         <v>129549.25</v>
       </c>
-      <c r="K29" s="29" t="s">
+      <c r="K29" s="23" t="s">
         <v>87</v>
       </c>
-      <c r="P29" s="13"/>
-      <c r="Q29" s="13"/>
-      <c r="R29" s="13"/>
-      <c r="S29" s="13"/>
     </row>
     <row r="30" spans="1:19">
       <c r="A30" t="s">
@@ -4576,17 +4507,13 @@
       <c r="H30">
         <v>0</v>
       </c>
-      <c r="I30" s="5">
+      <c r="I30" s="4">
         <f>32966*0.3</f>
         <v>9889.7999999999993</v>
       </c>
-      <c r="K30" s="29" t="s">
+      <c r="K30" s="23" t="s">
         <v>87</v>
       </c>
-      <c r="P30" s="13"/>
-      <c r="Q30" s="13"/>
-      <c r="R30" s="13"/>
-      <c r="S30" s="13"/>
     </row>
     <row r="31" spans="1:19">
       <c r="A31" t="s">
@@ -4607,59 +4534,45 @@
       <c r="H31">
         <v>0</v>
       </c>
-      <c r="I31" s="5">
+      <c r="I31" s="4">
         <f>196581*0.3</f>
         <v>58974.299999999996</v>
       </c>
-      <c r="K31" s="29" t="s">
+      <c r="K31" s="23" t="s">
         <v>87</v>
       </c>
-      <c r="P31" s="13"/>
-      <c r="Q31" s="13"/>
-      <c r="R31" s="13"/>
-      <c r="S31" s="13"/>
     </row>
     <row r="32" spans="1:19">
-      <c r="K32" s="6"/>
-      <c r="P32" s="13"/>
-      <c r="Q32" s="13"/>
-      <c r="R32" s="13"/>
-      <c r="S32" s="13"/>
-    </row>
-    <row r="33" spans="1:19">
-      <c r="P33" s="13"/>
-      <c r="Q33" s="12"/>
-      <c r="R33" s="12"/>
-      <c r="S33" s="13"/>
-    </row>
-    <row r="34" spans="1:19">
-      <c r="A34" s="7" t="s">
+      <c r="K32" s="3"/>
+    </row>
+    <row r="33" spans="1:18">
+      <c r="Q33" s="10"/>
+      <c r="R33" s="10"/>
+    </row>
+    <row r="34" spans="1:18">
+      <c r="A34" s="5" t="s">
         <v>138</v>
       </c>
-      <c r="P34" s="13"/>
-      <c r="Q34" s="12"/>
-      <c r="R34" s="12"/>
-      <c r="S34" s="13"/>
-    </row>
-    <row r="35" spans="1:19">
+      <c r="Q34" s="10"/>
+      <c r="R34" s="10"/>
+    </row>
+    <row r="35" spans="1:18">
       <c r="A35" s="1" t="s">
         <v>134</v>
       </c>
-      <c r="K35" s="19" t="s">
+      <c r="K35" s="14" t="s">
         <v>135</v>
       </c>
-      <c r="L35" s="20" t="s">
+      <c r="L35" s="15" t="s">
         <v>136</v>
       </c>
-      <c r="M35" s="21" t="s">
+      <c r="M35" s="16" t="s">
         <v>137</v>
       </c>
-      <c r="P35" s="13"/>
-      <c r="Q35" s="12"/>
-      <c r="R35" s="12"/>
-      <c r="S35" s="13"/>
-    </row>
-    <row r="36" spans="1:19">
+      <c r="Q35" s="10"/>
+      <c r="R35" s="10"/>
+    </row>
+    <row r="36" spans="1:18">
       <c r="A36" t="s">
         <v>95</v>
       </c>
@@ -4682,21 +4595,17 @@
         <f t="shared" ref="I36:I45" si="0">MIN(MAX(H36*$K$36,$L$36),$M$36)</f>
         <v>35</v>
       </c>
-      <c r="K36" s="24">
+      <c r="K36" s="19">
         <v>3</v>
       </c>
-      <c r="L36" s="22">
+      <c r="L36" s="17">
         <v>35</v>
       </c>
-      <c r="M36" s="23">
+      <c r="M36" s="18">
         <v>100</v>
       </c>
-      <c r="P36" s="13"/>
-      <c r="Q36" s="13"/>
-      <c r="R36" s="13"/>
-      <c r="S36" s="13"/>
-    </row>
-    <row r="37" spans="1:19">
+    </row>
+    <row r="37" spans="1:18">
       <c r="A37" t="s">
         <v>97</v>
       </c>
@@ -4720,7 +4629,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="38" spans="1:19">
+    <row r="38" spans="1:18">
       <c r="A38" t="s">
         <v>98</v>
       </c>
@@ -4743,11 +4652,11 @@
         <f t="shared" si="0"/>
         <v>35</v>
       </c>
-      <c r="K38" s="28" t="s">
+      <c r="K38" s="22" t="s">
         <v>148</v>
       </c>
     </row>
-    <row r="39" spans="1:19">
+    <row r="39" spans="1:18">
       <c r="A39" t="s">
         <v>99</v>
       </c>
@@ -4771,7 +4680,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="40" spans="1:19">
+    <row r="40" spans="1:18">
       <c r="A40" t="s">
         <v>100</v>
       </c>
@@ -4795,7 +4704,7 @@
         <v>38.099999999999994</v>
       </c>
     </row>
-    <row r="41" spans="1:19">
+    <row r="41" spans="1:18">
       <c r="A41" t="s">
         <v>101</v>
       </c>
@@ -4819,7 +4728,7 @@
         <v>38.099999999999994</v>
       </c>
     </row>
-    <row r="42" spans="1:19">
+    <row r="42" spans="1:18">
       <c r="A42" t="s">
         <v>102</v>
       </c>
@@ -4843,7 +4752,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="43" spans="1:19">
+    <row r="43" spans="1:18">
       <c r="A43" t="s">
         <v>103</v>
       </c>
@@ -4867,7 +4776,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="44" spans="1:19">
+    <row r="44" spans="1:18">
       <c r="A44" t="s">
         <v>104</v>
       </c>
@@ -4891,7 +4800,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="45" spans="1:19">
+    <row r="45" spans="1:18">
       <c r="A45" t="s">
         <v>105</v>
       </c>
@@ -4915,12 +4824,12 @@
         <v>35</v>
       </c>
     </row>
-    <row r="46" spans="1:19">
+    <row r="46" spans="1:18">
       <c r="A46" s="1" t="s">
         <v>106</v>
       </c>
     </row>
-    <row r="47" spans="1:19">
+    <row r="47" spans="1:18">
       <c r="A47" t="s">
         <v>107</v>
       </c>
@@ -4944,7 +4853,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="48" spans="1:19">
+    <row r="48" spans="1:18">
       <c r="A48" t="s">
         <v>108</v>
       </c>
@@ -5618,7 +5527,7 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:L47"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
@@ -5678,10 +5587,10 @@
       <c r="H2">
         <v>1</v>
       </c>
-      <c r="J2" s="3">
+      <c r="J2" s="2">
         <v>1.4</v>
       </c>
-      <c r="L2" s="28" t="s">
+      <c r="L2" s="22" t="s">
         <v>145</v>
       </c>
     </row>
@@ -5701,10 +5610,10 @@
       <c r="H3">
         <v>1</v>
       </c>
-      <c r="J3" s="3">
+      <c r="J3" s="2">
         <v>1.4</v>
       </c>
-      <c r="L3" s="28" t="s">
+      <c r="L3" s="22" t="s">
         <v>146</v>
       </c>
     </row>
@@ -5724,7 +5633,7 @@
       <c r="H4">
         <v>1</v>
       </c>
-      <c r="J4" s="3">
+      <c r="J4" s="2">
         <v>1.36</v>
       </c>
     </row>
@@ -5744,7 +5653,7 @@
       <c r="H5">
         <v>1</v>
       </c>
-      <c r="J5" s="3">
+      <c r="J5" s="2">
         <v>1.33</v>
       </c>
     </row>
@@ -5764,7 +5673,7 @@
       <c r="H6">
         <v>1</v>
       </c>
-      <c r="J6" s="3">
+      <c r="J6" s="2">
         <v>1.33</v>
       </c>
     </row>
@@ -5784,7 +5693,7 @@
       <c r="H7">
         <v>1</v>
       </c>
-      <c r="J7" s="3">
+      <c r="J7" s="2">
         <v>1.36</v>
       </c>
     </row>
@@ -5804,7 +5713,7 @@
       <c r="H8">
         <v>1</v>
       </c>
-      <c r="J8" s="3">
+      <c r="J8" s="2">
         <v>1.36</v>
       </c>
     </row>
@@ -5824,7 +5733,7 @@
       <c r="H9">
         <v>1</v>
       </c>
-      <c r="J9" s="3">
+      <c r="J9" s="2">
         <v>1.36</v>
       </c>
     </row>
@@ -5844,7 +5753,7 @@
       <c r="H10">
         <v>1</v>
       </c>
-      <c r="J10" s="3">
+      <c r="J10" s="2">
         <v>1</v>
       </c>
     </row>
@@ -5864,7 +5773,7 @@
       <c r="H11">
         <v>1</v>
       </c>
-      <c r="J11" s="3">
+      <c r="J11" s="2">
         <v>1.32</v>
       </c>
     </row>
@@ -5884,7 +5793,7 @@
       <c r="H12">
         <v>1</v>
       </c>
-      <c r="J12" s="3">
+      <c r="J12" s="2">
         <v>1.35</v>
       </c>
     </row>
@@ -5904,7 +5813,7 @@
       <c r="H13">
         <v>1</v>
       </c>
-      <c r="J13" s="3">
+      <c r="J13" s="2">
         <v>1.35</v>
       </c>
     </row>
@@ -5924,7 +5833,7 @@
       <c r="H14">
         <v>1</v>
       </c>
-      <c r="J14" s="3">
+      <c r="J14" s="2">
         <v>1.33</v>
       </c>
     </row>
@@ -5944,7 +5853,7 @@
       <c r="H15">
         <v>1</v>
       </c>
-      <c r="J15" s="3">
+      <c r="J15" s="2">
         <v>1.32</v>
       </c>
     </row>
@@ -5964,7 +5873,7 @@
       <c r="H16">
         <v>1</v>
       </c>
-      <c r="J16" s="3">
+      <c r="J16" s="2">
         <v>1.32</v>
       </c>
     </row>
@@ -5984,7 +5893,7 @@
       <c r="H17">
         <v>1</v>
       </c>
-      <c r="J17" s="3">
+      <c r="J17" s="2">
         <v>1.38</v>
       </c>
     </row>
@@ -6004,7 +5913,7 @@
       <c r="H18">
         <v>1</v>
       </c>
-      <c r="J18" s="3">
+      <c r="J18" s="2">
         <v>1.38</v>
       </c>
     </row>
@@ -6024,7 +5933,7 @@
       <c r="H20">
         <v>1</v>
       </c>
-      <c r="J20" s="3">
+      <c r="J20" s="2">
         <v>1.45</v>
       </c>
     </row>
@@ -6044,7 +5953,7 @@
       <c r="H21">
         <v>1</v>
       </c>
-      <c r="J21" s="3">
+      <c r="J21" s="2">
         <v>1.45</v>
       </c>
     </row>
@@ -6064,7 +5973,7 @@
       <c r="H22">
         <v>1</v>
       </c>
-      <c r="J22" s="3">
+      <c r="J22" s="2">
         <v>1.64</v>
       </c>
     </row>
@@ -6084,7 +5993,7 @@
       <c r="H23">
         <v>1</v>
       </c>
-      <c r="J23" s="3">
+      <c r="J23" s="2">
         <v>1.33</v>
       </c>
     </row>
@@ -6104,7 +6013,7 @@
       <c r="H24">
         <v>1</v>
       </c>
-      <c r="J24" s="3">
+      <c r="J24" s="2">
         <v>1.33</v>
       </c>
     </row>
@@ -6124,7 +6033,7 @@
       <c r="H25">
         <v>1</v>
       </c>
-      <c r="J25" s="3">
+      <c r="J25" s="2">
         <v>1.35</v>
       </c>
     </row>
@@ -6144,7 +6053,7 @@
       <c r="H26">
         <v>1</v>
       </c>
-      <c r="J26" s="3">
+      <c r="J26" s="2">
         <v>1.37</v>
       </c>
     </row>
@@ -6164,7 +6073,7 @@
       <c r="H27">
         <v>1</v>
       </c>
-      <c r="J27" s="3">
+      <c r="J27" s="2">
         <v>1.37</v>
       </c>
     </row>
@@ -6184,7 +6093,7 @@
       <c r="H28">
         <v>1</v>
       </c>
-      <c r="J28" s="3">
+      <c r="J28" s="2">
         <v>1.32</v>
       </c>
     </row>
@@ -6204,7 +6113,7 @@
       <c r="H29">
         <v>1</v>
       </c>
-      <c r="J29" s="3">
+      <c r="J29" s="2">
         <v>1</v>
       </c>
     </row>
@@ -6224,7 +6133,7 @@
       <c r="H30">
         <v>1</v>
       </c>
-      <c r="J30" s="3">
+      <c r="J30" s="2">
         <v>1.34</v>
       </c>
     </row>
@@ -6244,7 +6153,7 @@
       <c r="H31">
         <v>1</v>
       </c>
-      <c r="J31" s="3">
+      <c r="J31" s="2">
         <v>1.34</v>
       </c>
     </row>
@@ -6264,7 +6173,7 @@
       <c r="H32">
         <v>1</v>
       </c>
-      <c r="J32" s="3">
+      <c r="J32" s="2">
         <v>1</v>
       </c>
     </row>
@@ -6284,7 +6193,7 @@
       <c r="H33">
         <v>1</v>
       </c>
-      <c r="J33" s="3">
+      <c r="J33" s="2">
         <v>1.54</v>
       </c>
     </row>
@@ -6304,7 +6213,7 @@
       <c r="H34">
         <v>1</v>
       </c>
-      <c r="J34" s="3">
+      <c r="J34" s="2">
         <v>1.54</v>
       </c>
     </row>
@@ -6324,7 +6233,7 @@
       <c r="H35">
         <v>1</v>
       </c>
-      <c r="J35" s="3">
+      <c r="J35" s="2">
         <v>1.38</v>
       </c>
     </row>
@@ -6344,7 +6253,7 @@
       <c r="H36">
         <v>1</v>
       </c>
-      <c r="J36" s="3">
+      <c r="J36" s="2">
         <v>1.38</v>
       </c>
     </row>
@@ -6364,7 +6273,7 @@
       <c r="H38">
         <v>100</v>
       </c>
-      <c r="I38" s="9">
+      <c r="I38" s="7">
         <v>8</v>
       </c>
     </row>
@@ -6384,7 +6293,7 @@
       <c r="H39">
         <v>100</v>
       </c>
-      <c r="I39" s="9">
+      <c r="I39" s="7">
         <v>15</v>
       </c>
     </row>
@@ -6404,7 +6313,7 @@
       <c r="H40">
         <v>100</v>
       </c>
-      <c r="J40" s="9">
+      <c r="J40" s="7">
         <v>100</v>
       </c>
     </row>
@@ -6424,7 +6333,7 @@
       <c r="H41">
         <v>100</v>
       </c>
-      <c r="J41" s="9">
+      <c r="J41" s="7">
         <v>100</v>
       </c>
     </row>
@@ -6458,23 +6367,23 @@
       <c r="H44">
         <v>0</v>
       </c>
-      <c r="J44" s="25">
-        <v>17</v>
-      </c>
-      <c r="L44" s="28" t="s">
+      <c r="J44" s="8">
+        <v>10</v>
+      </c>
+      <c r="L44" s="22" t="s">
         <v>160</v>
       </c>
     </row>
     <row r="45" spans="2:12">
-      <c r="L45" s="28"/>
+      <c r="L45" s="22"/>
     </row>
     <row r="46" spans="2:12">
-      <c r="H46" s="31"/>
-      <c r="I46" s="31"/>
-      <c r="J46" s="31"/>
+      <c r="H46" s="11"/>
+      <c r="I46" s="11"/>
+      <c r="J46" s="11"/>
     </row>
     <row r="47" spans="2:12">
-      <c r="I47" s="26"/>
+      <c r="I47" s="20"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -6483,7 +6392,7 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:I16"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
@@ -6524,10 +6433,10 @@
       </c>
     </row>
     <row r="2" spans="1:9">
-      <c r="A2" s="7" t="s">
+      <c r="A2" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="B2" s="7"/>
+      <c r="B2" s="5"/>
     </row>
     <row r="3" spans="1:9">
       <c r="A3" t="s">
@@ -6628,10 +6537,10 @@
       <c r="F8" t="s">
         <v>60</v>
       </c>
-      <c r="G8" s="4" t="s">
+      <c r="G8" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="H8" s="4">
+      <c r="H8" s="3">
         <v>1</v>
       </c>
       <c r="I8">
@@ -6645,10 +6554,10 @@
       <c r="F9" t="s">
         <v>60</v>
       </c>
-      <c r="G9" s="4" t="s">
+      <c r="G9" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="H9" s="4">
+      <c r="H9" s="3">
         <v>1</v>
       </c>
       <c r="I9">
@@ -6656,109 +6565,109 @@
       </c>
     </row>
     <row r="11" spans="1:9">
-      <c r="E11" s="4" t="s">
+      <c r="E11" s="3" t="s">
         <v>54</v>
       </c>
-      <c r="F11" s="4" t="s">
+      <c r="F11" s="3" t="s">
         <v>55</v>
       </c>
-      <c r="G11" s="4" t="s">
+      <c r="G11" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="H11" s="4">
-        <v>1</v>
-      </c>
-      <c r="I11" s="4">
+      <c r="H11" s="3">
+        <v>1</v>
+      </c>
+      <c r="I11" s="3">
         <f>AVERAGE(1.33,1.31)</f>
         <v>1.32</v>
       </c>
     </row>
     <row r="12" spans="1:9">
-      <c r="E12" s="4" t="s">
+      <c r="E12" s="3" t="s">
         <v>56</v>
       </c>
-      <c r="F12" s="4" t="s">
+      <c r="F12" s="3" t="s">
         <v>55</v>
       </c>
-      <c r="G12" s="4" t="s">
+      <c r="G12" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="H12" s="4">
-        <v>1</v>
-      </c>
-      <c r="I12" s="4">
+      <c r="H12" s="3">
+        <v>1</v>
+      </c>
+      <c r="I12" s="3">
         <f t="shared" ref="I12:I16" si="0">AVERAGE(1.33,1.31)</f>
         <v>1.32</v>
       </c>
     </row>
     <row r="13" spans="1:9">
-      <c r="E13" s="4" t="s">
+      <c r="E13" s="3" t="s">
         <v>57</v>
       </c>
-      <c r="F13" s="4" t="s">
+      <c r="F13" s="3" t="s">
         <v>55</v>
       </c>
-      <c r="G13" s="4" t="s">
+      <c r="G13" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="H13" s="4">
-        <v>1</v>
-      </c>
-      <c r="I13" s="4">
+      <c r="H13" s="3">
+        <v>1</v>
+      </c>
+      <c r="I13" s="3">
         <f t="shared" si="0"/>
         <v>1.32</v>
       </c>
     </row>
     <row r="14" spans="1:9">
-      <c r="E14" s="4" t="s">
+      <c r="E14" s="3" t="s">
         <v>54</v>
       </c>
       <c r="F14" t="s">
         <v>59</v>
       </c>
-      <c r="G14" s="4" t="s">
+      <c r="G14" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="H14" s="4">
-        <v>1</v>
-      </c>
-      <c r="I14" s="4">
+      <c r="H14" s="3">
+        <v>1</v>
+      </c>
+      <c r="I14" s="3">
         <f t="shared" si="0"/>
         <v>1.32</v>
       </c>
     </row>
     <row r="15" spans="1:9">
-      <c r="E15" s="4" t="s">
+      <c r="E15" s="3" t="s">
         <v>56</v>
       </c>
       <c r="F15" t="s">
         <v>59</v>
       </c>
-      <c r="G15" s="4" t="s">
+      <c r="G15" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="H15" s="4">
-        <v>1</v>
-      </c>
-      <c r="I15" s="4">
+      <c r="H15" s="3">
+        <v>1</v>
+      </c>
+      <c r="I15" s="3">
         <f t="shared" si="0"/>
         <v>1.32</v>
       </c>
     </row>
     <row r="16" spans="1:9">
-      <c r="E16" s="4" t="s">
+      <c r="E16" s="3" t="s">
         <v>57</v>
       </c>
       <c r="F16" t="s">
         <v>59</v>
       </c>
-      <c r="G16" s="4" t="s">
+      <c r="G16" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="H16" s="4">
-        <v>1</v>
-      </c>
-      <c r="I16" s="4">
+      <c r="H16" s="3">
+        <v>1</v>
+      </c>
+      <c r="I16" s="3">
         <f t="shared" si="0"/>
         <v>1.32</v>
       </c>
@@ -6769,7 +6678,7 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="A1:H2"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
@@ -6814,7 +6723,7 @@
       <c r="F2">
         <v>1.25</v>
       </c>
-      <c r="H2" s="28" t="s">
+      <c r="H2" s="22" t="s">
         <v>149</v>
       </c>
     </row>
@@ -6825,7 +6734,7 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
   <dimension ref="A1:H3"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
@@ -6868,7 +6777,7 @@
       <c r="F2">
         <v>1.27</v>
       </c>
-      <c r="H2" s="28" t="s">
+      <c r="H2" s="22" t="s">
         <v>149</v>
       </c>
     </row>
@@ -6888,7 +6797,7 @@
       <c r="F3">
         <v>0.9</v>
       </c>
-      <c r="H3" s="28" t="s">
+      <c r="H3" s="22" t="s">
         <v>150</v>
       </c>
     </row>
@@ -6898,7 +6807,7 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
   <dimension ref="A1:F2"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
@@ -6932,7 +6841,7 @@
       <c r="D2">
         <v>1.1499999999999999</v>
       </c>
-      <c r="F2" s="28" t="s">
+      <c r="F2" s="22" t="s">
         <v>149</v>
       </c>
     </row>
@@ -6942,7 +6851,7 @@
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0700-000000000000}">
   <dimension ref="A1:F16"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
@@ -7219,7 +7128,7 @@
 </file>
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0800-000000000000}">
   <dimension ref="A1:N46"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
@@ -7260,188 +7169,188 @@
       <c r="F2">
         <v>53</v>
       </c>
-      <c r="H2" s="28" t="s">
+      <c r="H2" s="22" t="s">
         <v>93</v>
       </c>
     </row>
     <row r="3" spans="1:14">
-      <c r="H3" s="28" t="s">
+      <c r="H3" s="22" t="s">
         <v>92</v>
       </c>
     </row>
     <row r="4" spans="1:14">
-      <c r="B4" s="33"/>
-      <c r="H4" s="28" t="s">
+      <c r="B4" s="26"/>
+      <c r="H4" s="22" t="s">
         <v>151</v>
       </c>
     </row>
     <row r="5" spans="1:14">
-      <c r="B5" s="33"/>
+      <c r="B5" s="26"/>
     </row>
     <row r="6" spans="1:14">
-      <c r="B6" s="33"/>
-      <c r="N6" s="32"/>
+      <c r="B6" s="26"/>
+      <c r="N6" s="25"/>
     </row>
     <row r="7" spans="1:14">
-      <c r="B7" s="33"/>
-      <c r="N7" s="32"/>
+      <c r="B7" s="26"/>
+      <c r="N7" s="25"/>
     </row>
     <row r="8" spans="1:14">
-      <c r="B8" s="33"/>
-      <c r="N8" s="32"/>
+      <c r="B8" s="26"/>
+      <c r="N8" s="25"/>
     </row>
     <row r="9" spans="1:14">
-      <c r="B9" s="33"/>
-      <c r="N9" s="32"/>
+      <c r="B9" s="26"/>
+      <c r="N9" s="25"/>
     </row>
     <row r="10" spans="1:14">
-      <c r="B10" s="33"/>
-      <c r="N10" s="32"/>
+      <c r="B10" s="26"/>
+      <c r="N10" s="25"/>
     </row>
     <row r="11" spans="1:14">
-      <c r="B11" s="33"/>
-      <c r="N11" s="32"/>
+      <c r="B11" s="26"/>
+      <c r="N11" s="25"/>
     </row>
     <row r="12" spans="1:14">
-      <c r="B12" s="33"/>
-      <c r="N12" s="32"/>
+      <c r="B12" s="26"/>
+      <c r="N12" s="25"/>
     </row>
     <row r="13" spans="1:14">
-      <c r="B13" s="33"/>
-      <c r="N13" s="32"/>
+      <c r="B13" s="26"/>
+      <c r="N13" s="25"/>
     </row>
     <row r="14" spans="1:14">
-      <c r="B14" s="33"/>
-      <c r="N14" s="32"/>
+      <c r="B14" s="26"/>
+      <c r="N14" s="25"/>
     </row>
     <row r="15" spans="1:14">
-      <c r="B15" s="33"/>
-      <c r="N15" s="32"/>
+      <c r="B15" s="26"/>
+      <c r="N15" s="25"/>
     </row>
     <row r="16" spans="1:14">
-      <c r="B16" s="33"/>
-      <c r="N16" s="32"/>
+      <c r="B16" s="26"/>
+      <c r="N16" s="25"/>
     </row>
     <row r="17" spans="2:14">
-      <c r="B17" s="33"/>
-      <c r="N17" s="32"/>
+      <c r="B17" s="26"/>
+      <c r="N17" s="25"/>
     </row>
     <row r="18" spans="2:14">
-      <c r="B18" s="33"/>
-      <c r="N18" s="32"/>
+      <c r="B18" s="26"/>
+      <c r="N18" s="25"/>
     </row>
     <row r="19" spans="2:14">
-      <c r="B19" s="33"/>
-      <c r="N19" s="32"/>
+      <c r="B19" s="26"/>
+      <c r="N19" s="25"/>
     </row>
     <row r="20" spans="2:14">
-      <c r="B20" s="33"/>
-      <c r="N20" s="32"/>
+      <c r="B20" s="26"/>
+      <c r="N20" s="25"/>
     </row>
     <row r="21" spans="2:14">
-      <c r="B21" s="33"/>
-      <c r="N21" s="32"/>
+      <c r="B21" s="26"/>
+      <c r="N21" s="25"/>
     </row>
     <row r="22" spans="2:14">
-      <c r="B22" s="33"/>
-      <c r="N22" s="32"/>
+      <c r="B22" s="26"/>
+      <c r="N22" s="25"/>
     </row>
     <row r="23" spans="2:14">
-      <c r="B23" s="33"/>
-      <c r="N23" s="32"/>
+      <c r="B23" s="26"/>
+      <c r="N23" s="25"/>
     </row>
     <row r="24" spans="2:14">
-      <c r="B24" s="33"/>
-      <c r="N24" s="32"/>
+      <c r="B24" s="26"/>
+      <c r="N24" s="25"/>
     </row>
     <row r="25" spans="2:14">
-      <c r="B25" s="33"/>
-      <c r="N25" s="32"/>
+      <c r="B25" s="26"/>
+      <c r="N25" s="25"/>
     </row>
     <row r="26" spans="2:14">
-      <c r="B26" s="33"/>
-      <c r="N26" s="32"/>
+      <c r="B26" s="26"/>
+      <c r="N26" s="25"/>
     </row>
     <row r="27" spans="2:14">
-      <c r="B27" s="33"/>
-      <c r="N27" s="32"/>
+      <c r="B27" s="26"/>
+      <c r="N27" s="25"/>
     </row>
     <row r="28" spans="2:14">
-      <c r="B28" s="33"/>
-      <c r="N28" s="32"/>
+      <c r="B28" s="26"/>
+      <c r="N28" s="25"/>
     </row>
     <row r="29" spans="2:14">
-      <c r="B29" s="33"/>
-      <c r="N29" s="32"/>
+      <c r="B29" s="26"/>
+      <c r="N29" s="25"/>
     </row>
     <row r="30" spans="2:14">
-      <c r="B30" s="33"/>
-      <c r="N30" s="32"/>
+      <c r="B30" s="26"/>
+      <c r="N30" s="25"/>
     </row>
     <row r="31" spans="2:14">
-      <c r="B31" s="33"/>
-      <c r="N31" s="32"/>
+      <c r="B31" s="26"/>
+      <c r="N31" s="25"/>
     </row>
     <row r="32" spans="2:14">
-      <c r="B32" s="33"/>
-      <c r="N32" s="32"/>
+      <c r="B32" s="26"/>
+      <c r="N32" s="25"/>
     </row>
     <row r="33" spans="2:14">
-      <c r="B33" s="33"/>
-      <c r="N33" s="32"/>
+      <c r="B33" s="26"/>
+      <c r="N33" s="25"/>
     </row>
     <row r="34" spans="2:14">
-      <c r="B34" s="33"/>
-      <c r="N34" s="32"/>
+      <c r="B34" s="26"/>
+      <c r="N34" s="25"/>
     </row>
     <row r="35" spans="2:14">
-      <c r="B35" s="33"/>
-      <c r="N35" s="32"/>
+      <c r="B35" s="26"/>
+      <c r="N35" s="25"/>
     </row>
     <row r="36" spans="2:14">
-      <c r="B36" s="33"/>
-      <c r="N36" s="32"/>
+      <c r="B36" s="26"/>
+      <c r="N36" s="25"/>
     </row>
     <row r="37" spans="2:14">
-      <c r="B37" s="33"/>
-      <c r="N37" s="32"/>
+      <c r="B37" s="26"/>
+      <c r="N37" s="25"/>
     </row>
     <row r="38" spans="2:14">
-      <c r="B38" s="33"/>
-      <c r="N38" s="32"/>
+      <c r="B38" s="26"/>
+      <c r="N38" s="25"/>
     </row>
     <row r="39" spans="2:14">
-      <c r="B39" s="33"/>
-      <c r="N39" s="32"/>
+      <c r="B39" s="26"/>
+      <c r="N39" s="25"/>
     </row>
     <row r="40" spans="2:14">
-      <c r="B40" s="33"/>
-      <c r="N40" s="32"/>
+      <c r="B40" s="26"/>
+      <c r="N40" s="25"/>
     </row>
     <row r="41" spans="2:14">
-      <c r="B41" s="33"/>
-      <c r="N41" s="32"/>
+      <c r="B41" s="26"/>
+      <c r="N41" s="25"/>
     </row>
     <row r="42" spans="2:14">
-      <c r="B42" s="33"/>
-      <c r="N42" s="32"/>
+      <c r="B42" s="26"/>
+      <c r="N42" s="25"/>
     </row>
     <row r="43" spans="2:14">
-      <c r="B43" s="33"/>
-      <c r="N43" s="32"/>
+      <c r="B43" s="26"/>
+      <c r="N43" s="25"/>
     </row>
     <row r="44" spans="2:14">
-      <c r="B44" s="33"/>
-      <c r="N44" s="32"/>
+      <c r="B44" s="26"/>
+      <c r="N44" s="25"/>
     </row>
     <row r="45" spans="2:14">
-      <c r="N45" s="32"/>
+      <c r="N45" s="25"/>
     </row>
     <row r="46" spans="2:14">
-      <c r="N46" s="32"/>
+      <c r="N46" s="25"/>
     </row>
   </sheetData>
-  <sortState ref="A4:F40">
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A4:F40">
     <sortCondition ref="B4:B40"/>
   </sortState>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Corrected minor typo in Sust50 scenario definition
</commit_message>
<xml_diff>
--- a/data/scenarios/example_org_circ.xlsx
+++ b/data/scenarios/example_org_circ.xlsx
@@ -1,11 +1,11 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28623"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29029"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{28BAE003-BE4D-4216-BCD8-506D76E50C25}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{15387E32-9A44-4914-A058-09A98E879386}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-38520" yWindow="-120" windowWidth="38640" windowHeight="21120" tabRatio="746" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-38520" yWindow="-120" windowWidth="38640" windowHeight="21120" tabRatio="746" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Regions" sheetId="11" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1047" uniqueCount="161">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1047" uniqueCount="160">
   <si>
     <t>val_is</t>
   </si>
@@ -411,9 +411,6 @@
   </si>
   <si>
     <t>Offals</t>
-  </si>
-  <si>
-    <t>share_imported</t>
   </si>
   <si>
     <t>Blood in food</t>
@@ -1058,7 +1055,7 @@
   <sheetData>
     <row r="1" spans="1:13">
       <c r="A1" s="1" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>38</v>
@@ -1084,7 +1081,7 @@
     </row>
     <row r="3" spans="1:13">
       <c r="K3" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="L3">
         <v>0.01</v>
@@ -1092,7 +1089,7 @@
     </row>
     <row r="4" spans="1:13">
       <c r="K4" s="5" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
     </row>
     <row r="5" spans="1:13">
@@ -1106,7 +1103,7 @@
         <v>1011</v>
       </c>
       <c r="E5" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="F5" t="s">
         <v>36</v>
@@ -1122,7 +1119,7 @@
         <v>25594.738467494699</v>
       </c>
       <c r="M5" s="24" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
     </row>
     <row r="6" spans="1:13">
@@ -1136,7 +1133,7 @@
         <v>111</v>
       </c>
       <c r="E6" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="F6" t="s">
         <v>36</v>
@@ -1152,7 +1149,7 @@
         <v>30470.923931982899</v>
       </c>
       <c r="M6" s="24" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
     </row>
     <row r="7" spans="1:13">
@@ -1166,7 +1163,7 @@
         <v>1111</v>
       </c>
       <c r="E7" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="F7" t="s">
         <v>36</v>
@@ -1182,7 +1179,7 @@
         <v>29995.316181367401</v>
       </c>
       <c r="M7" s="24" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
     </row>
     <row r="8" spans="1:13">
@@ -1196,7 +1193,7 @@
         <v>1112</v>
       </c>
       <c r="E8" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="F8" t="s">
         <v>36</v>
@@ -1212,7 +1209,7 @@
         <v>20762.5598364898</v>
       </c>
       <c r="M8" s="24" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
     </row>
     <row r="9" spans="1:13">
@@ -1226,7 +1223,7 @@
         <v>112</v>
       </c>
       <c r="E9" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="F9" t="s">
         <v>36</v>
@@ -1253,7 +1250,7 @@
         <v>1121</v>
       </c>
       <c r="E10" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="F10" t="s">
         <v>36</v>
@@ -1280,7 +1277,7 @@
         <v>1122</v>
       </c>
       <c r="E11" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="F11" t="s">
         <v>36</v>
@@ -1307,7 +1304,7 @@
         <v>1123</v>
       </c>
       <c r="E12" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="F12" t="s">
         <v>36</v>
@@ -1334,7 +1331,7 @@
         <v>1124</v>
       </c>
       <c r="E13" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="F13" t="s">
         <v>36</v>
@@ -1361,7 +1358,7 @@
         <v>1131</v>
       </c>
       <c r="E14" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="F14" t="s">
         <v>36</v>
@@ -1388,7 +1385,7 @@
         <v>1211</v>
       </c>
       <c r="E15" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="F15" t="s">
         <v>36</v>
@@ -1415,7 +1412,7 @@
         <v>1212</v>
       </c>
       <c r="E16" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="F16" t="s">
         <v>36</v>
@@ -1442,7 +1439,7 @@
         <v>1213</v>
       </c>
       <c r="E17" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="F17" t="s">
         <v>36</v>
@@ -1469,7 +1466,7 @@
         <v>1214</v>
       </c>
       <c r="E18" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="F18" t="s">
         <v>36</v>
@@ -1496,7 +1493,7 @@
         <v>1215</v>
       </c>
       <c r="E19" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="F19" t="s">
         <v>36</v>
@@ -1523,7 +1520,7 @@
         <v>1216</v>
       </c>
       <c r="E20" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="F20" t="s">
         <v>36</v>
@@ -1550,7 +1547,7 @@
         <v>1221</v>
       </c>
       <c r="E21" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="F21" t="s">
         <v>36</v>
@@ -1577,7 +1574,7 @@
         <v>1222</v>
       </c>
       <c r="E22" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="F22" t="s">
         <v>36</v>
@@ -1604,7 +1601,7 @@
         <v>1311</v>
       </c>
       <c r="E23" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="F23" t="s">
         <v>36</v>
@@ -1631,7 +1628,7 @@
         <v>1321</v>
       </c>
       <c r="E24" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="F24" t="s">
         <v>36</v>
@@ -1658,7 +1655,7 @@
         <v>1322</v>
       </c>
       <c r="E25" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="F25" t="s">
         <v>36</v>
@@ -1685,7 +1682,7 @@
         <v>1331</v>
       </c>
       <c r="E26" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="F26" t="s">
         <v>36</v>
@@ -1712,7 +1709,7 @@
         <v>1411</v>
       </c>
       <c r="E27" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="F27" t="s">
         <v>36</v>
@@ -1739,7 +1736,7 @@
         <v>1412</v>
       </c>
       <c r="E28" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="F28" t="s">
         <v>36</v>
@@ -1766,7 +1763,7 @@
         <v>1421</v>
       </c>
       <c r="E29" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="F29" t="s">
         <v>36</v>
@@ -1793,7 +1790,7 @@
         <v>1511</v>
       </c>
       <c r="E30" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="F30" t="s">
         <v>36</v>
@@ -1820,7 +1817,7 @@
         <v>1512</v>
       </c>
       <c r="E31" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="F31" t="s">
         <v>36</v>
@@ -1847,7 +1844,7 @@
         <v>1521</v>
       </c>
       <c r="E32" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="F32" t="s">
         <v>36</v>
@@ -1874,7 +1871,7 @@
         <v>1522</v>
       </c>
       <c r="E33" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="F33" t="s">
         <v>36</v>
@@ -1901,7 +1898,7 @@
         <v>1611</v>
       </c>
       <c r="E34" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="F34" t="s">
         <v>36</v>
@@ -1928,7 +1925,7 @@
         <v>1612</v>
       </c>
       <c r="E35" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="F35" t="s">
         <v>36</v>
@@ -1955,7 +1952,7 @@
         <v>1613</v>
       </c>
       <c r="E36" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="F36" t="s">
         <v>36</v>
@@ -1982,7 +1979,7 @@
         <v>1614</v>
       </c>
       <c r="E37" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="F37" t="s">
         <v>36</v>
@@ -2009,7 +2006,7 @@
         <v>1615</v>
       </c>
       <c r="E38" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="F38" t="s">
         <v>36</v>
@@ -2036,7 +2033,7 @@
         <v>1616</v>
       </c>
       <c r="E39" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="F39" t="s">
         <v>36</v>
@@ -2063,7 +2060,7 @@
         <v>1617</v>
       </c>
       <c r="E40" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="F40" t="s">
         <v>36</v>
@@ -2090,7 +2087,7 @@
         <v>1621</v>
       </c>
       <c r="E41" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="F41" t="s">
         <v>36</v>
@@ -2117,7 +2114,7 @@
         <v>1622</v>
       </c>
       <c r="E42" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="F42" t="s">
         <v>36</v>
@@ -2144,7 +2141,7 @@
         <v>1623</v>
       </c>
       <c r="E43" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="F43" t="s">
         <v>36</v>
@@ -2171,7 +2168,7 @@
         <v>1711</v>
       </c>
       <c r="E44" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="F44" t="s">
         <v>36</v>
@@ -2198,7 +2195,7 @@
         <v>1712</v>
       </c>
       <c r="E45" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="F45" t="s">
         <v>36</v>
@@ -2225,7 +2222,7 @@
         <v>1713</v>
       </c>
       <c r="E46" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="F46" t="s">
         <v>36</v>
@@ -2252,7 +2249,7 @@
         <v>1721</v>
       </c>
       <c r="E47" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="F47" t="s">
         <v>36</v>
@@ -2279,7 +2276,7 @@
         <v>1722</v>
       </c>
       <c r="E48" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="F48" t="s">
         <v>36</v>
@@ -2306,7 +2303,7 @@
         <v>1723</v>
       </c>
       <c r="E49" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="F49" t="s">
         <v>36</v>
@@ -2333,7 +2330,7 @@
         <v>1724</v>
       </c>
       <c r="E50" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="F50" t="s">
         <v>36</v>
@@ -2360,7 +2357,7 @@
         <v>1811</v>
       </c>
       <c r="E51" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="F51" t="s">
         <v>36</v>
@@ -2387,7 +2384,7 @@
         <v>1812</v>
       </c>
       <c r="E52" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="F52" t="s">
         <v>36</v>
@@ -2414,7 +2411,7 @@
         <v>1813</v>
       </c>
       <c r="E53" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="F53" t="s">
         <v>36</v>
@@ -2441,7 +2438,7 @@
         <v>1821</v>
       </c>
       <c r="E54" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="F54" t="s">
         <v>36</v>
@@ -2468,7 +2465,7 @@
         <v>1911</v>
       </c>
       <c r="E55" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="F55" t="s">
         <v>36</v>
@@ -2495,7 +2492,7 @@
         <v>1912</v>
       </c>
       <c r="E56" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="F56" t="s">
         <v>36</v>
@@ -2522,7 +2519,7 @@
         <v>1921</v>
       </c>
       <c r="E57" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="F57" t="s">
         <v>36</v>
@@ -2549,7 +2546,7 @@
         <v>1922</v>
       </c>
       <c r="E58" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="F58" t="s">
         <v>36</v>
@@ -2576,7 +2573,7 @@
         <v>2011</v>
       </c>
       <c r="E59" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="F59" t="s">
         <v>36</v>
@@ -2603,7 +2600,7 @@
         <v>2012</v>
       </c>
       <c r="E60" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="F60" t="s">
         <v>36</v>
@@ -2630,7 +2627,7 @@
         <v>2019</v>
       </c>
       <c r="E61" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="F61" t="s">
         <v>36</v>
@@ -2657,7 +2654,7 @@
         <v>2111</v>
       </c>
       <c r="E62" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="F62" t="s">
         <v>36</v>
@@ -2684,7 +2681,7 @@
         <v>2121</v>
       </c>
       <c r="E63" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="F63" t="s">
         <v>36</v>
@@ -2711,7 +2708,7 @@
         <v>2122</v>
       </c>
       <c r="E64" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="F64" t="s">
         <v>36</v>
@@ -2738,7 +2735,7 @@
         <v>2211</v>
       </c>
       <c r="E65" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="F65" t="s">
         <v>36</v>
@@ -2765,7 +2762,7 @@
         <v>2212</v>
       </c>
       <c r="E66" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="F66" t="s">
         <v>36</v>
@@ -2792,7 +2789,7 @@
         <v>2221</v>
       </c>
       <c r="E67" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="F67" t="s">
         <v>36</v>
@@ -2819,7 +2816,7 @@
         <v>2311</v>
       </c>
       <c r="E68" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="F68" t="s">
         <v>36</v>
@@ -2846,7 +2843,7 @@
         <v>2312</v>
       </c>
       <c r="E69" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="F69" t="s">
         <v>36</v>
@@ -2873,7 +2870,7 @@
         <v>2319</v>
       </c>
       <c r="E70" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="F70" t="s">
         <v>36</v>
@@ -2900,7 +2897,7 @@
         <v>2331</v>
       </c>
       <c r="E71" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="F71" t="s">
         <v>36</v>
@@ -2927,7 +2924,7 @@
         <v>2411</v>
       </c>
       <c r="E72" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="F72" t="s">
         <v>36</v>
@@ -2954,7 +2951,7 @@
         <v>2412</v>
       </c>
       <c r="E73" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="F73" t="s">
         <v>36</v>
@@ -2981,7 +2978,7 @@
         <v>2413</v>
       </c>
       <c r="E74" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="F74" t="s">
         <v>36</v>
@@ -3008,7 +3005,7 @@
         <v>2414</v>
       </c>
       <c r="E75" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="F75" t="s">
         <v>36</v>
@@ -3035,7 +3032,7 @@
         <v>2415</v>
       </c>
       <c r="E76" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="F76" t="s">
         <v>36</v>
@@ -3062,7 +3059,7 @@
         <v>2419</v>
       </c>
       <c r="E77" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="F77" t="s">
         <v>36</v>
@@ -3089,7 +3086,7 @@
         <v>2511</v>
       </c>
       <c r="E78" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="F78" t="s">
         <v>36</v>
@@ -3116,7 +3113,7 @@
         <v>2512</v>
       </c>
       <c r="E79" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="F79" t="s">
         <v>36</v>
@@ -3143,7 +3140,7 @@
         <v>2519</v>
       </c>
       <c r="E80" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="F80" t="s">
         <v>36</v>
@@ -3170,7 +3167,7 @@
         <v>2521</v>
       </c>
       <c r="E81" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="F81" t="s">
         <v>36</v>
@@ -3197,7 +3194,7 @@
         <v>311</v>
       </c>
       <c r="E82" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="F82" t="s">
         <v>36</v>
@@ -3224,7 +3221,7 @@
         <v>312</v>
       </c>
       <c r="E83" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="F83" t="s">
         <v>36</v>
@@ -3251,7 +3248,7 @@
         <v>321</v>
       </c>
       <c r="E84" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="F84" t="s">
         <v>36</v>
@@ -3278,7 +3275,7 @@
         <v>322</v>
       </c>
       <c r="E85" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="F85" t="s">
         <v>36</v>
@@ -3305,7 +3302,7 @@
         <v>411</v>
       </c>
       <c r="E86" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="F86" t="s">
         <v>36</v>
@@ -3332,7 +3329,7 @@
         <v>421</v>
       </c>
       <c r="E87" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="F87" t="s">
         <v>36</v>
@@ -3359,7 +3356,7 @@
         <v>422</v>
       </c>
       <c r="E88" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="F88" t="s">
         <v>36</v>
@@ -3386,7 +3383,7 @@
         <v>431</v>
       </c>
       <c r="E89" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="F89" t="s">
         <v>36</v>
@@ -3413,7 +3410,7 @@
         <v>511</v>
       </c>
       <c r="E90" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="F90" t="s">
         <v>36</v>
@@ -3440,7 +3437,7 @@
         <v>512</v>
       </c>
       <c r="E91" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="F91" t="s">
         <v>36</v>
@@ -3467,7 +3464,7 @@
         <v>513</v>
       </c>
       <c r="E92" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="F92" t="s">
         <v>36</v>
@@ -3494,7 +3491,7 @@
         <v>514</v>
       </c>
       <c r="E93" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="F93" t="s">
         <v>36</v>
@@ -3521,7 +3518,7 @@
         <v>515</v>
       </c>
       <c r="E94" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="F94" t="s">
         <v>36</v>
@@ -3548,7 +3545,7 @@
         <v>521</v>
       </c>
       <c r="E95" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="F95" t="s">
         <v>36</v>
@@ -3575,7 +3572,7 @@
         <v>611</v>
       </c>
       <c r="E96" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="F96" t="s">
         <v>36</v>
@@ -3602,7 +3599,7 @@
         <v>612</v>
       </c>
       <c r="E97" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="F97" t="s">
         <v>36</v>
@@ -3629,7 +3626,7 @@
         <v>621</v>
       </c>
       <c r="E98" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="F98" t="s">
         <v>36</v>
@@ -3656,7 +3653,7 @@
         <v>622</v>
       </c>
       <c r="E99" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="F99" t="s">
         <v>36</v>
@@ -3683,7 +3680,7 @@
         <v>711</v>
       </c>
       <c r="E100" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="F100" t="s">
         <v>36</v>
@@ -3710,7 +3707,7 @@
         <v>731</v>
       </c>
       <c r="E101" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="F101" t="s">
         <v>36</v>
@@ -3737,7 +3734,7 @@
         <v>811</v>
       </c>
       <c r="E102" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="F102" t="s">
         <v>36</v>
@@ -3764,7 +3761,7 @@
         <v>812</v>
       </c>
       <c r="E103" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="F103" t="s">
         <v>36</v>
@@ -3791,7 +3788,7 @@
         <v>813</v>
       </c>
       <c r="E104" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="F104" t="s">
         <v>36</v>
@@ -3818,7 +3815,7 @@
         <v>814</v>
       </c>
       <c r="E105" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="F105" t="s">
         <v>36</v>
@@ -3845,7 +3842,7 @@
         <v>821</v>
       </c>
       <c r="E106" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="F106" t="s">
         <v>36</v>
@@ -3872,7 +3869,7 @@
         <v>831</v>
       </c>
       <c r="E107" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="F107" t="s">
         <v>36</v>
@@ -3899,7 +3896,7 @@
         <v>911</v>
       </c>
       <c r="E108" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="F108" t="s">
         <v>36</v>
@@ -3926,7 +3923,7 @@
         <v>912</v>
       </c>
       <c r="E109" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="F109" t="s">
         <v>36</v>
@@ -3953,7 +3950,7 @@
         <v>913</v>
       </c>
       <c r="E110" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="F110" t="s">
         <v>36</v>
@@ -3997,7 +3994,7 @@
         <v>22</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="D1" s="1" t="s">
         <v>3</v>
@@ -4458,7 +4455,7 @@
         <v>87</v>
       </c>
       <c r="M28" s="22" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
     </row>
     <row r="29" spans="1:19">
@@ -4551,23 +4548,23 @@
     </row>
     <row r="34" spans="1:18">
       <c r="A34" s="5" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="Q34" s="10"/>
       <c r="R34" s="10"/>
     </row>
     <row r="35" spans="1:18">
       <c r="A35" s="1" t="s">
+        <v>133</v>
+      </c>
+      <c r="K35" s="14" t="s">
         <v>134</v>
       </c>
-      <c r="K35" s="14" t="s">
+      <c r="L35" s="15" t="s">
         <v>135</v>
       </c>
-      <c r="L35" s="15" t="s">
+      <c r="M35" s="16" t="s">
         <v>136</v>
-      </c>
-      <c r="M35" s="16" t="s">
-        <v>137</v>
       </c>
       <c r="Q35" s="10"/>
       <c r="R35" s="10"/>
@@ -4653,7 +4650,7 @@
         <v>35</v>
       </c>
       <c r="K38" s="22" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
     </row>
     <row r="39" spans="1:18">
@@ -5304,7 +5301,7 @@
         <v>8</v>
       </c>
       <c r="F70" t="s">
-        <v>124</v>
+        <v>9</v>
       </c>
       <c r="G70" t="s">
         <v>36</v>
@@ -5319,7 +5316,7 @@
     </row>
     <row r="71" spans="1:9">
       <c r="A71" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="C71" t="s">
         <v>96</v>
@@ -5328,7 +5325,7 @@
         <v>8</v>
       </c>
       <c r="F71" t="s">
-        <v>124</v>
+        <v>9</v>
       </c>
       <c r="G71" t="s">
         <v>36</v>
@@ -5372,7 +5369,7 @@
     </row>
     <row r="74" spans="1:9">
       <c r="A74" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="C74" t="s">
         <v>96</v>
@@ -5396,7 +5393,7 @@
     </row>
     <row r="75" spans="1:9">
       <c r="A75" s="1" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
     </row>
     <row r="76" spans="1:9">
@@ -5422,7 +5419,7 @@
     </row>
     <row r="77" spans="1:9">
       <c r="A77" s="1" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
     </row>
     <row r="78" spans="1:9">
@@ -5451,12 +5448,12 @@
     </row>
     <row r="79" spans="1:9">
       <c r="A79" s="1" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
     </row>
     <row r="80" spans="1:9">
       <c r="A80" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="D80" t="s">
         <v>8</v>
@@ -5477,7 +5474,7 @@
     </row>
     <row r="81" spans="1:9">
       <c r="A81" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="D81" t="s">
         <v>8</v>
@@ -5498,7 +5495,7 @@
     </row>
     <row r="82" spans="1:9">
       <c r="A82" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="D82" t="s">
         <v>8</v>
@@ -5550,7 +5547,7 @@
         <v>38</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="E1" s="1" t="s">
         <v>3</v>
@@ -5565,7 +5562,7 @@
         <v>7</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="J1" s="1" t="s">
         <v>16</v>
@@ -5591,7 +5588,7 @@
         <v>1.4</v>
       </c>
       <c r="L2" s="22" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
     </row>
     <row r="3" spans="1:12">
@@ -5614,7 +5611,7 @@
         <v>1.4</v>
       </c>
       <c r="L3" s="22" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
     </row>
     <row r="4" spans="1:12">
@@ -6259,13 +6256,13 @@
     </row>
     <row r="38" spans="2:12">
       <c r="D38" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="E38" t="s">
         <v>8</v>
       </c>
       <c r="F38" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="G38" t="s">
         <v>24</v>
@@ -6279,13 +6276,13 @@
     </row>
     <row r="39" spans="2:12">
       <c r="D39" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="E39" t="s">
         <v>8</v>
       </c>
       <c r="F39" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="G39" t="s">
         <v>24</v>
@@ -6299,13 +6296,13 @@
     </row>
     <row r="40" spans="2:12">
       <c r="D40" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="E40" t="s">
         <v>6</v>
       </c>
       <c r="F40" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="G40" t="s">
         <v>24</v>
@@ -6319,13 +6316,13 @@
     </row>
     <row r="41" spans="2:12">
       <c r="D41" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="E41" t="s">
         <v>6</v>
       </c>
       <c r="F41" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="G41" t="s">
         <v>24</v>
@@ -6342,7 +6339,7 @@
         <v>6</v>
       </c>
       <c r="F43" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="G43" t="s">
         <v>24</v>
@@ -6359,7 +6356,7 @@
         <v>8</v>
       </c>
       <c r="F44" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="G44" t="s">
         <v>24</v>
@@ -6371,7 +6368,7 @@
         <v>10</v>
       </c>
       <c r="L44" s="22" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
     </row>
     <row r="45" spans="2:12">
@@ -6724,7 +6721,7 @@
         <v>1.25</v>
       </c>
       <c r="H2" s="22" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
     </row>
   </sheetData>
@@ -6778,7 +6775,7 @@
         <v>1.27</v>
       </c>
       <c r="H2" s="22" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
     </row>
     <row r="3" spans="1:8">
@@ -6798,7 +6795,7 @@
         <v>0.9</v>
       </c>
       <c r="H3" s="22" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
     </row>
   </sheetData>
@@ -6842,7 +6839,7 @@
         <v>1.1499999999999999</v>
       </c>
       <c r="F2" s="22" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
     </row>
   </sheetData>
@@ -7181,7 +7178,7 @@
     <row r="4" spans="1:14">
       <c r="B4" s="26"/>
       <c r="H4" s="22" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
     </row>
     <row r="5" spans="1:14">

</xml_diff>